<commit_message>
Improve scraper by fixing real-time log output
Update scraper start endpoint to use unbuffered Python execution for real-time log streaming and ensure environment variables are correctly set.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 166d9f9e-4654-4c30-a21d-c31f51b6ad9a
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 769961e7-9f03-4446-8d5f-7f5bad53f019
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/a20dc0d8-683e-46b6-8c48-962056d15fa0/166d9f9e-4654-4c30-a21d-c31f51b6ad9a/SUVCXPU
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backup_temp.xlsx
+++ b/backup_temp.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H451"/>
+  <dimension ref="A1:H551"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16878,6 +16878,3622 @@
         </is>
       </c>
     </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>Rika For Computer</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>01221645635</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>01221645635</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr"/>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>22 El Rakhaa St., El zawia el hamra, Cairo, EL ZAWIA EL HAMRA</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/566036</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2B Egypt</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr"/>
+      <c r="C453" t="inlineStr"/>
+      <c r="D453" t="inlineStr"/>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>218 Faisal St., El Taawon, Faisal, Giza, FAISAL</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/713221</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>Forbed</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr"/>
+      <c r="C454" t="inlineStr"/>
+      <c r="D454" t="inlineStr"/>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>Old Market, Quwasnah, El monofeya, QUWASNAH</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/713097</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>Gouda</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>01228867246</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>01228867246</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr"/>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>53 El Ahrar St., Shoubra el khaymah, Kaliobeya, SHOUBRA EL KHAYMAH</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/414888</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>Abou Aly For Printers</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>01115050733</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>01115050733</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr"/>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>Mahaleya 6, , 1st District, Obour city, Kaliobeya, OBOUR CITY</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/525938</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>O Bounto</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>01003275394</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>01003275394</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr"/>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>El Lawandy St., Shoubra el khaymah, Kaliobeya, SHOUBRA EL KHAYMAH</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/418224</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>0237814706</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr"/>
+      <c r="D458" t="inlineStr"/>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>18 Fahmy Hegazy St., Faisal, Giza, FAISAL</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>الميكانيكا</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/393832</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>El Rebh El Basit Furniture</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>01225414630</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>01225414630</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr"/>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>3 Geziret Badran St., Shoubra, Cairo, SHOUBRA</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/434543</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>El Faranseya For Computer Maintenance</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>01142471246</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>01142471246</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr"/>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>3 Atteya El Sawalhy St., Off Makram Ebaid St., 8th District, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/483444</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>KBH Solutions - Facilities Management</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>01090337497</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>01090337497</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr"/>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>6 Ragaa Abdel Rasoul St., Off Wadi El Nil St., Mohandeseen, Giza, MOHANDESEEN</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>أدوات النظافة</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/429188</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>Saber Net</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>01146192030</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>01146192030</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr"/>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>5 Salama El Wefy St., Zahraa Ain Shams, Ain shams el sharkeya, Cairo, AIN SHAMS EL SHARKEYA</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/478888</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>El Haj Gomaa &amp; Sons Furniture</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>01126502505</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>01126502505</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr"/>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>17 Wabor El Teheen St., El bassateen, Cairo, EL BASSATEEN</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/504929</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>El Safa For Modern Furniture</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>01111423260</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>01111423260</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr"/>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>16 Soliman Salem St., El Dawagen, Helwan, Cairo, HELWAN</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/461008</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>Compu Royal</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>0553777738</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr"/>
+      <c r="D465" t="inlineStr"/>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>El Shafaey St., Deyerb negm, El sharkeya, DEYERB NEGM</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/330983</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>Arab Engineers</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>01009994062</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>01009994062</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr"/>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>18 El Bostan St., Bab el louk, Cairo, BAB EL LOUK</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/618261</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>El Sohagy For Coffee Shop Supplies</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>01121835500</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>01121835500</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr"/>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>38 El Bosta St., Geziret Mohamed Village, El warak, Giza, EL WARAK</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+        </is>
+      </c>
+      <c r="G467" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/599141</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>Compu Magic</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>01117587400</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>01117587400</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr"/>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>Mekka El Mokarrama St.  1St Neighbourhood, 7th District, 6th of october, Giza, 6th OF OCTOBER</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/438409</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>Ema For Services &amp; Suppling</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>01280005706</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>01280005706</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr"/>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>35 El Faraby St., 1st Compound, New cairo, Cairo, NEW CAIRO</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>أدوات النظافة</t>
+        </is>
+      </c>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/495777</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>Infasme</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>0224191555</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr"/>
+      <c r="D470" t="inlineStr"/>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>97 Omar Ibn El Khattab St., Floor 5, El Sabaa Emarat Sq., Almaza, Heliopolis, Cairo, HELIOPOLIS</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/440508</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>Malek Furniture</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>0237710916</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr"/>
+      <c r="D471" t="inlineStr"/>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>Faisal St.  Intersection Of El Mariouteya St., El Mariouteya, El haram, Giza, EL HARAM</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/508565</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>Creative For General Supplies</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>01028494985</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>01028494985</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr"/>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>1 El Moahda St., Plaza Tower, El mansoura, El dakahleya, EL MANSOURA</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/706113</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>Nazih Refaat El Ais</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>0225109894</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr"/>
+      <c r="D473" t="inlineStr"/>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>El Ghoureya St., Azhar, Cairo, AZHAR</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/384470</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>No Name Furniture</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>01004780139</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>01004780139</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr"/>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>5 Hussein Sherin St., Loran, Alexandria, LORAN</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/470367</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>El Azaly Furniture</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>01116640735</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>01116640735</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr"/>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>El Azaly St.  Off Saad Zaghloul St., El hawamdeya, Giza, EL HAWAMDEYA</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/373862</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>El Kilany For Electronics Maintenance</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>01212887317</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>01212887317</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr"/>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>4 Alaa El Din St., Bashteel Village, Auseem, Giza, AUSEEM</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>الإلكترونيات</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/542290</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>One Thing For Computer</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>01553954397</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>01553954397</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr"/>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>El Sabaq St., Heliopolis, Cairo, HELIOPOLIS</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/670439</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>Grand Furniture</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>01234555598</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>01234555598</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr"/>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>44 Makram Ebaid St., Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/707353</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>Forbed</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr"/>
+      <c r="C479" t="inlineStr"/>
+      <c r="D479" t="inlineStr"/>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>El Thalathiny St., Abou Gabal Sq., Dayrut, Assyout, DAYRUT</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/713278</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>Professional Health &amp; Safety Establishment</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>0225911117</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr"/>
+      <c r="D480" t="inlineStr"/>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>7   El Kabara Alley, Off El Gomhoureya St., Downtown, Cairo, DOWNTOWN</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>الصحة والسلامة ومقاومة الحريق</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/568743</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>Sanabel For Electronics</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>01228506460</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>01228506460</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr"/>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>31 Mahmoud Ammar St.  Off El Warsha St., 8th District, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>الإلكترونيات</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/310163</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr"/>
+      <c r="C482" t="inlineStr"/>
+      <c r="D482" t="inlineStr"/>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>40 El Mansoureya St., El gamaleya, Cairo, EL GAMALEYA</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>الإلكترونيات</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/633368</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>Target For Import And Export</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>01110444615</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>01110444615</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr"/>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>, 1St Industrial Zone, El katameya, Cairo, EL KATAMEYA</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/685213</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>El Maktb El Masry</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>01001090568</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>01001090568</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr"/>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>Ahmed Eissa St., Qalyub, Kaliobeya, QALYUB</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>الميكانيكا</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/601986</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>On Wood Furniture</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>01100690161</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>01100690161</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr"/>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>, 2nd Industrial Zone, Kom ushim, El fayoum, KOM USHIM</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/621650</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>Hub Furniture</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr"/>
+      <c r="C486" t="inlineStr"/>
+      <c r="D486" t="inlineStr"/>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>Omar Ibn El Khattab St., Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/627292</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>Fawry Plus</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr"/>
+      <c r="C487" t="inlineStr"/>
+      <c r="D487" t="inlineStr"/>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>Plot 18, Block 6 El Taqqa St., 8th District, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>الإلكترونيات</t>
+        </is>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/633632</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>X Treme For Computer</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>01226601352</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>01226601352</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr"/>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>3 Atteya El Sawalhy St., Extension Of Makram Ebaid St., 8th District, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/599670</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>Mido For Computer</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>01062745216</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>01062745216</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr"/>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>10 El Taawoneyat Bldgs., El Galaa El Bahary St., Shebein el kawm, El monofeya, SHEBEIN EL KAWM</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/544017</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>Values Home</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr"/>
+      <c r="C490" t="inlineStr"/>
+      <c r="D490" t="inlineStr"/>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>1 Makram Ebaid St., Floor 4, City Light Tower, 6th Zone, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/559365</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>El Andalus For Computer</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>01015956001</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>01015956001</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr"/>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>2 Hussein El Sheikh Aly St., Kerdasa, Giza, Kerdasa</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G491" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H491" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/557817</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>Jana</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>01280283470</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>01280283470</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr"/>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>8 Abdel Sattar El Hawary St., Ain shams, Cairo, AIN SHAMS</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/420822</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>El Hoda Center</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>01113752279</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>01113752279</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr"/>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>El Ansary St., Boulak el dakrour, Giza, BOULAK EL DAKROUR</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/339971</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>El Mokhtar For Computer Maintenance</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>01061804950</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>01061804950</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr"/>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>18 El Bostan St., Bab el louk, Cairo, BAB EL LOUK</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/546053</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>Game City Play Station</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>01229062404</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>01229062404</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr"/>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>8 El Deeb St., Minuf, El monofeya, MINUF</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/571379</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>El Qasr El Domyaty</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>01006731506</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>01006731506</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr"/>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>6 El Gesr El Barrany St., Dar el salam, Cairo, DAR EL SALAM</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/329176</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>Sphinx &amp; El Ahram For Lifting Furniture</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>01201188700</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>01201188700</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr"/>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>El Estad St., Tanta, El gharbeya, TANTA</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/463653</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>El Masreyeen For Electrical Supplies</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>0225748483</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr"/>
+      <c r="D498" t="inlineStr"/>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>16 Zakareya Ahmed St., El Tawfiqeya, Downtown, Cairo, DOWNTOWN</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/388555</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>El Arabya Co. For Furniture</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>01022000235</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>01022000235</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr"/>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>76 El Wehda El Arabeya St., Gesr el suez, Cairo, GESR EL SUEZ</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/576834</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>El Qenawy</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>01225020815</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>01225020815</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr"/>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>El Souk St., Samannoud, El gharbeya, SAMANNOUD</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/345479</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>Tiba</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>01090650650</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>01090650650</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr"/>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>El Thanawy El Aam St., Aboul matamir, El beheira, ABOUL MATAMIR</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/374703</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>Hammad Computer Center</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>01008778851</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>01008778851</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr"/>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>Ahmed Maher St., Mit ghamr, El dakahleya, MIT GHAMR</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/669664</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>El Bait Furniture</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>01225830046</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>01225830046</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr"/>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>Saad Zaghloul St., Belbeis, El sharkeya, BELBEIS</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/324535</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>Green Emp</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>0220650337</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr"/>
+      <c r="D504" t="inlineStr"/>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>27 El Moltaqa El Araby St., Floor 1, Sheraton Bldgs., Heliopolis, Cairo, HELIOPOLIS</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>الميكانيكا</t>
+        </is>
+      </c>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/633926</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>El Rabea For Computer</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>01208082525</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>01208082525</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr"/>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>1 El Sagha St., Ashmoun, El monofeya, ASHMOUN</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G505" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/560191</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>Angle American Furniture</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>01006446634</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>01006446634</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr"/>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>, 4th Neighbourhood, El Motamayez District, 6th of october, Giza, 6th OF OCTOBER</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/485629</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>Delta For Integrated Industries</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr"/>
+      <c r="C507" t="inlineStr"/>
+      <c r="D507" t="inlineStr"/>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>9 Omar Ibn Abdel Aziz St., Assyout, Assyout, Assyout</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>أدوات النظافة</t>
+        </is>
+      </c>
+      <c r="G507" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/708128</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>Mada Holding</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>0225057546</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr"/>
+      <c r="D508" t="inlineStr"/>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>55 El Ashgar St., Plot 8058, Mokattam, Cairo, MOKATTAM</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/515906</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>El Mansour Furniture</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>01026471144</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>01026471144</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr"/>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>10 B Hassan El Maamoun St., Floor 1, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G509" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/679048</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>Bavarian Play Staion</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>01221379610</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>01221379610</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr"/>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>2, Haridy Alley, Faisal, Giza, FAISAL</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/685128</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>Dominoes Code</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>0236678080</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr"/>
+      <c r="D511" t="inlineStr"/>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>1723 Rd. 40  8th Neighbourhood, 3rd District, 6th of october, Giza, 6th OF OCTOBER</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G511" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/539602</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>El Gallad Group</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>01222228844</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>01222228844</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr"/>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>Plot 348, , Industrial Zone, 5th Compound, New cairo, Cairo, NEW CAIRO</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/581112</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>El Amal Fire Doors</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>01121351446</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>01121351446</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr"/>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>, El Manayel Village, Kafr Hamza -Abo Zaabal, El khanka, Kaliobeya, EL KHANKA</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>الصحة والسلامة ومقاومة الحريق</t>
+        </is>
+      </c>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/698650</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>Extra Light</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>0225778075</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr"/>
+      <c r="D514" t="inlineStr"/>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>18 Zakareya Ahmed St.  Off Emad El Din St., El Tawfiqeya, Downtown, Cairo, DOWNTOWN</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/570880</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>Malaket El Zaitoun For Furniture</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>01225918848</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>01225918848</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr"/>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>53 Metwally El Waseef St., Ezbet el nakhl, Cairo, EZBET EL NAKHL</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/533267</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>Capital Plus</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>01224781111</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>01224781111</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr"/>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>Shebin El Koum St., Downtown, Ismaileya, DOWNTOWN</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>الصحة والسلامة ومقاومة الحريق</t>
+        </is>
+      </c>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/711173</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>Fawry Plus</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr"/>
+      <c r="C517" t="inlineStr"/>
+      <c r="D517" t="inlineStr"/>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>51 El Gomhoureya St., Samalut, El menia, SAMALUT</t>
+        </is>
+      </c>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>الإلكترونيات</t>
+        </is>
+      </c>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/698251</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>International Academy For Studies &amp; Computer</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>01003859782</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>01003859782</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr"/>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>El Gomhoureya St., As-santah, El gharbeya, AS-SANTAH</t>
+        </is>
+      </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/349627</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>Casper</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>0226265309</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr"/>
+      <c r="D519" t="inlineStr"/>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>Souk El Wadi St., Spico, El salam city, Cairo, EL SALAM CITY</t>
+        </is>
+      </c>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G519" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/441348</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>Kasr El Ahlam</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>01092334411</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>01092334411</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr"/>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>Maaneya Rd., Etay el barod, El beheira, ETAY EL BAROD</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G520" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/371281</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>M &amp; S Technology</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>01003496303</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>01003496303</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr"/>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>64 El Farahda St., Al laban, Alexandria, AL LABAN</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>الميكانيكا</t>
+        </is>
+      </c>
+      <c r="G521" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/581900</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>Mohamed Soliman For Computer</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>01116081002</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>01116081002</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr"/>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>1 El Nahda St., El hawamdeya, Giza, EL HAWAMDEYA</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G522" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/603715</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>Technology For Computer Accessories</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>01143675390</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>01143675390</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr"/>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>137 Moassaset El Zakah St., El marg, Cairo, EL MARG</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G523" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/624242</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>Giga Byte For Computer</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>01093080074</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>01093080074</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr"/>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>9 Beacho American City Bldgs. Abdel Rahman Ibn Auf St., Phase 1, Zahraa El Maadi, Maadi, Cairo, MAADI</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G524" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/537133</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>G.Tech</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>0222579572</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr"/>
+      <c r="D525" t="inlineStr"/>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>7 Sphinx Sq., Mohandeseen, Giza, MOHANDESEEN</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G525" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/449583</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>El Sewedy Power Cables</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>01002240142</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>01002240142</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr"/>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>92 Mohamed Naguib St., Ataba, Cairo, ATABA</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="G526" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/708900</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>National Steam Boiler</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>01097920066</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>01097920066</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr"/>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>Cairo Belbeis Desert Rd., El Tayara Sq., 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>الميكانيكا</t>
+        </is>
+      </c>
+      <c r="G527" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/706248</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>Sabry Showroom For Furniture</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>01225632434</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>01225632434</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr"/>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>2 Sabry El Halawany St., El marg, Cairo, EL MARG</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G528" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/484863</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>Free Net Cafe</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>0224341087</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr"/>
+      <c r="D529" t="inlineStr"/>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>10 El Sheikh El Zarqany St., Hadayek el kobba, Cairo, HADAYEK EL KOBBA</t>
+        </is>
+      </c>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G529" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H529" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/419906</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>Select Training &amp; Technology Solutions</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>0502200498</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr"/>
+      <c r="D530" t="inlineStr"/>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>26 El Gomhoureya St., El mansoura, El dakahleya, EL MANSOURA</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G530" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/532744</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>Unix Note Books</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>0224518786</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr"/>
+      <c r="D531" t="inlineStr"/>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>9 El Sakhawy St., Mansheyet El Bakry, Heliopolis, Cairo, HELIOPOLIS</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G531" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H531" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/545665</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>Shift For Information Technology Services</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>0226221884</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr"/>
+      <c r="D532" t="inlineStr"/>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>11 El Nasr St., El nozha el gadida, Cairo, EL NOZHA EL GADIDA</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G532" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/458729</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>Infinity Egypt</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>01111116623</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>01111116623</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr"/>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>2 Hassan Afify St., Flat 63, Floor 6, Off Ahmed El Sawy St., El Safwa Tower, 6th Zone, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G533" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H533" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/600212</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>Professional For Computer Services</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>0223951783</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr"/>
+      <c r="D534" t="inlineStr"/>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>1, Opera Sq., Ataba, Cairo, ATABA</t>
+        </is>
+      </c>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G534" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H534" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/307871</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>El Nour For Furniture</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>01112144311</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>01112144311</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr"/>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>4 Rafea Abou El Ela El Hambouly St., El baragil, Giza, EL BARAGIL</t>
+        </is>
+      </c>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G535" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H535" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/561176</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>El Masreya For Language &amp; Computer</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>035294737</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr"/>
+      <c r="D536" t="inlineStr"/>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>57 El Galaa St., Victoria, Alexandria, VICTORIA</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G536" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H536" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/466007</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>Future Power</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>01281861008</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>01281861008</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr"/>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>, Zone 11, Sadat city, El monofeya, SADAT City</t>
+        </is>
+      </c>
+      <c r="F537" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="G537" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H537" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/708391</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr"/>
+      <c r="C538" t="inlineStr"/>
+      <c r="D538" t="inlineStr"/>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>Iskandar Ibrahim St., Miami, Alexandria, MIAMI</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>الإلكترونيات</t>
+        </is>
+      </c>
+      <c r="G538" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H538" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/632357</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>Number One</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>01062297433</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>01062297433</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr"/>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>El Wehda St., Kerdasa, Giza, Kerdasa</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G539" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H539" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/362430</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>True Tech</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>01110505500</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>01110505500</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr"/>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>28 el estad st., Tanta, El gharbeya, TANTA</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G540" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/331971</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>Hosam For Computer Services</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>01062982975</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>01062982975</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr"/>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>19 El Eslah St.  Off El Kholafaa El Rashedin St., El khosous, Kaliobeya, EL KHOSOUS</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G541" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/495008</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>Game Spot</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>01226152461</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>01226152461</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr"/>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>11 El Marwa Bldgs. Nabil El Waqqad St., Ard El Golf, Heliopolis, Cairo, HELIOPOLIS</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G542" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H542" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/679260</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>Ahmed Moamen For Goods &amp; Furniture Transport</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>0572343223</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr"/>
+      <c r="D543" t="inlineStr"/>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>El Galaa St., Damietta, Damietta, DAMIETTA</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G543" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H543" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/381428</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>Digital Computer</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>0222756471</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr"/>
+      <c r="D544" t="inlineStr"/>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>28 Omar Lotfy St., Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G544" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/458238</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>Fiber One Systems</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>01201212574</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>01201212574</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr"/>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>615, Neighborhood 80, District 11, 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>الميكانيكا</t>
+        </is>
+      </c>
+      <c r="G545" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/662305</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>Cyber Tech</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>01110248186</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>01110248186</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr"/>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>4 El Adib Mohamed Zaitoun St., Semouha, Alexandria, SEMOUHA</t>
+        </is>
+      </c>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/470957</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr"/>
+      <c r="C547" t="inlineStr"/>
+      <c r="D547" t="inlineStr"/>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>80 El Eshreen St., Gesr el suez, Cairo, GESR EL SUEZ</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>الإلكترونيات</t>
+        </is>
+      </c>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/635841</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>Alam El Decor Showroom</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>01002778346</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>01002778346</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr"/>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>Luxor St., Imbaba, Giza, IMBABA</t>
+        </is>
+      </c>
+      <c r="F548" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G548" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/380881</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>New Special Office Furniture</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>0224041524</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr"/>
+      <c r="D549" t="inlineStr"/>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>50 El Nasr Rd., Extension Of Ramsis 2 St., Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G549" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/428462</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>Fawry Plus</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr"/>
+      <c r="C550" t="inlineStr"/>
+      <c r="D550" t="inlineStr"/>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>1 Ahmed Moharram St., El Saah Sq., Harb Tower, Damanhour, El beheira, Damanhour</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>الإلكترونيات</t>
+        </is>
+      </c>
+      <c r="G550" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/633480</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>Compu Center</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>01115829839</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>01115829839</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr"/>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>el gomhoureya st., Auseem, Giza, AUSEEM</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G551" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/349757</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Improve scraper progress reporting and phase detection
Adjusted the scraper to report progress every 200 requests instead of 1000, and refined phase detection logic in `scraper.ts` to accurately distinguish between YellowPages and Facebook phases. The `parseStats` function in `scraper.ts` was updated to correctly handle new log formats and prevent issues with zero companies found.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 2a1fad78-d05e-42f0-ad61-6fa4ea0cba54
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 1c25e72e-2d15-4e19-96d6-66a9c6eb084f
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/0ea4e3a5-1e4e-40d5-826b-5b1dabac3eb2/2a1fad78-d05e-42f0-ad61-6fa4ea0cba54/uCmf752
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backup_temp.xlsx
+++ b/backup_temp.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,28 +461,24 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Yehia For Electronics Repair</t>
+          <t>El Gamaa Center For Computer Maintenance</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>01005548672</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>01005548672</t>
-        </is>
-      </c>
+          <t>0133212997</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>17 Shahin St., Minuf, El monofeya, MINUF</t>
+          <t>30 Nassar St., Banha el gadida, Kaliobeya, BANHA EL GADIDA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>الإلكترونيات</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -492,30 +488,26 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/570597</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/520552</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>El Masry For Computer Maintenance</t>
+          <t>El Handasya For Supplies</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>01001322381</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>01001322381</t>
-        </is>
-      </c>
+          <t>0225175614</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>29 Khaled Ibn El Walid St., Ard El Gamaeya, Imbaba, Giza, IMBABA</t>
+          <t>9 W/4 Hassan Nassar St.  El Laselky Division, New Maadi, Maadi, Cairo, MAADI</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -530,35 +522,35 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/572012</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/428920</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ahlan 4 IT</t>
+          <t>El Nour El Mohamady Showroom</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>01111145958</t>
+          <t>01062670598</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>01111145958</t>
+          <t>01062670598</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>13 Dr. Mohamed Hassanein Heikal St., El mandara el bahareya, Alexandria, EL MANDARA EL BAHAREYA</t>
+          <t>56 El Nasr St., El maasara, Cairo, El Maasara</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -568,30 +560,30 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/620331</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/339870</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tito</t>
+          <t>El Mostaqbal</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>01229791682</t>
+          <t>01113276804</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>01229791682</t>
+          <t>01113276804</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2 Espico Bldgs.,, El salam city, Cairo, EL SALAM CITY</t>
+          <t>aly mubarak st., El Talbeya, El haram, Giza, EL HARAM</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -606,35 +598,35 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/389511</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/308602</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Al Adham Establishment For Supplies &amp; Refractories</t>
+          <t>Babmbo El Gharam</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01144997719</t>
+          <t>01222871263</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>01144997719</t>
+          <t>01222871263</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>6 El Nasr St.  Off Ard El Gamaeya St., Kozzika, Maadi, Cairo, MAADI</t>
+          <t>Samir Abdel Raouf St., Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -644,27 +636,35 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/440723</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/315410</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Games 2 Egypt</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
+          <t>Technical Workshop For Furniture</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>01278567502</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>01278567502</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7 Wadi El Nil St., Intersection Of Gamaet El Dewal El Arabeya St., Mohandeseen, Giza, MOHANDESEEN</t>
+          <t>5 Abou El Qassem Soliman St., El khosous, Kaliobeya, EL KHOSOUS</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -674,30 +674,30 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/651022</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/494395</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Shahd For Computer Service</t>
+          <t>El Alameya</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>01006212675</t>
+          <t>01226716304</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>01006212675</t>
+          <t>01226716304</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Damat Village, Kutour, El gharbeya, KUTOUR</t>
+          <t>El Sekka El Hadid St., Sayeda aisha, Cairo, SAYEDA AISHA</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -712,35 +712,27 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/552655</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/367996</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>El Kasr</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>01283509400</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>01283509400</t>
-        </is>
-      </c>
+          <t>Fawry Plus</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>El Salam St., Damanhour, El beheira, Damanhour</t>
+          <t>1 El Nabawy El Mohandes St., El Baraa Tower, El massalah, El fayoum, EL MASSALAH</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>الإلكترونيات</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -750,35 +742,35 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/361649</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/633492</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Smart Technology</t>
+          <t>El Loualoaa For Furniture</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>01222257827</t>
+          <t>01004001611</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>01222257827</t>
+          <t>01004001611</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Masged Abu El Naser St., Off El Samalihy 2 St., El bitash, Alexandria, EL BITASH</t>
+          <t>241 Ahmed Zaky St., Dar el salam, Cairo, DAR EL SALAM</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -788,35 +780,27 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/697257</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/477659</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>El Toubgy For Computer</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>01006803456</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>01006803456</t>
-        </is>
-      </c>
+          <t>Home Centre</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>60 El Khalifa El Maamoun St., Mansheyet El Bakry, Heliopolis, Cairo, HELIOPOLIS</t>
+          <t>Ring Rd., Cairo Festival City, New cairo, Cairo, NEW CAIRO</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -826,30 +810,26 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/621619</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/455082</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Arabia Furniture</t>
+          <t>On Time Establishment</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>01000358868</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>01000358868</t>
-        </is>
-      </c>
+          <t>0226273916</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>95 Mostafa El Nahhas St., Nasr city, Cairo, NASR CITY</t>
+          <t>Block 10, El Said A Bldgs., Belbeis Rd., El salam city, Cairo, EL SALAM CITY</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -864,31 +844,35 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/687066</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/333572</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Modern Systems Engineering</t>
+          <t>My Computer</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0224473103</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>01288004762</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>01288004762</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>3075 El Mostashar Hossam El Shamy St., El Mearag City, Zahraa El Maadi, Maadi, Cairo, MAADI</t>
+          <t>52 Lashin St., El Koum El Akhdar, Faisal, Giza, FAISAL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>الصحة والسلامة ومقاومة الحريق</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -898,35 +882,35 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/583830</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/398828</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Class For Furniture</t>
+          <t>Professional For Computer Services</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>01223926466</t>
+          <t>01119713080</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>01223926466</t>
+          <t>01119713080</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1St Industrial Zone, New damietta, Damietta, NEW DAMIETTA</t>
+          <t>5 El Marg El Omoumy St., El marg, Cairo, EL MARG</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -936,31 +920,35 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/590015</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/479341</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Retag For Trade &amp; Agencies</t>
+          <t>Ebdaa Furniture</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0222915859</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>01001916611</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>01001916611</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>66 El Nakhla El Motaey St., Triumph Square, Heliopolis, Cairo, HELIOPOLIS</t>
+          <t>30 El Galaa St., Damietta, Damietta, DAMIETTA</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -970,35 +958,35 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/414841</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/503176</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Compu Adham</t>
+          <t>Amada Steel For Metal Works And Forming</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>01285334014</t>
+          <t>01090650616</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>01285334014</t>
+          <t>01090650616</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>63 Selim St.  Off Faisal St., Faisal, Giza, FAISAL</t>
+          <t>13 El Madrasa St., Kafr Abou Seir, Moassaset el zakah, Cairo, MOASSASET EL ZAKAH</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1008,35 +996,35 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/392276</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/634156</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>El Haramain Showroom For Furniture</t>
+          <t>A2Z For Hotel &amp; Restaurant Supplies</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>01003883649</t>
+          <t>01224320350</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>01003883649</t>
+          <t>01224320350</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>el omda st., El Mariouteya, El haram, Giza, EL HARAM</t>
+          <t>6 El Masalla St., Flat 22, Floor 3, El Korba, Heliopolis, Cairo, HELIOPOLIS</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1046,31 +1034,35 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/328618</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/538523</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Atick Electronics</t>
+          <t>United International</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>034492883</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
+          <t>01115201602</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>01115201602</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>, Shakosh Village, Amreya, Alexandria, AMREYA</t>
+          <t>16 Mostafa El Sharqawy St., El herafeyeen, Cairo, EL HERAFEYEEN</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>الإلكترونيات</t>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1080,35 +1072,35 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/638309</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/373521</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>El Rabea Furniture</t>
+          <t>Sameh For Electronics</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>01270817413</t>
+          <t>01005223871</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>01270817413</t>
+          <t>01005223871</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2 Ahmed Hamdy St., El Monira El Gharbeya, Imbaba, Giza, IMBABA</t>
+          <t>Sherif St., Mit ghamr, El dakahleya, MIT GHAMR</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>الإلكترونيات</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1118,26 +1110,30 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/538901</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/339803</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Kasr Mohamed &amp; Amr</t>
+          <t>El Zaeem Furniture</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0238722575</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
+          <t>01118548660</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>01118548660</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>El Mansoureya St., El haram, Giza, EL HARAM</t>
+          <t>95 El Qalaa St., El sayeda zeinab, Cairo, EL SAYEDA ZEINAB</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1152,35 +1148,27 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/381345</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/649962</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Al Gehiny For Furniture &amp; Bedding</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>01200050039</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>01200050039</t>
-        </is>
-      </c>
+          <t>2B Egypt</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Mostafa Kamel Spine, Bldg. 7, 1st Compound, New cairo, Cairo, NEW CAIRO</t>
+          <t>6 Plot 363 Rd. 9, El Nafoura Sq., Mokattam, Cairo, MOKATTAM</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1190,35 +1178,35 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/485602</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/677942</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>National Steam Boiler</t>
+          <t>Star Pack</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>01091332366</t>
+          <t>01068900001</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>01091332366</t>
+          <t>01068900001</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Plot B5, Ebdaa Complex - 3rd Industrial Zone, 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
+          <t>El Kahrabaa St., Industrial Zone, Abou rawash, Giza, ABOU RAWASH</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>الميكانيكا</t>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1228,30 +1216,30 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/623342</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/638145</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Nada Tech</t>
+          <t>House Laser Printer</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>01224049904</t>
+          <t>01019373736</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>01224049904</t>
+          <t>01019373736</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>6 Zaid St., Off El Emam Mohamed Abdou St., Toril, El mansoura, El dakahleya, EL MANSOURA</t>
+          <t>50 El Khalifa El Maamoun St., Mansheyet El Bakry, Heliopolis, Cairo, HELIOPOLIS</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1266,31 +1254,35 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/652995</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/478106</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>El Hashemeya For Used Furniture</t>
+          <t>Volcano Center</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0226923253</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
+          <t>01090959990</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>01090959990</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Champs Elysees Passage, Commercial Market, Shop 249, Al rehab city, Cairo, AL REHAB CITY</t>
+          <t>Hassan El Badrawy St., Faisal, Giza, FAISAL</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1300,35 +1292,35 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/564066</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/418046</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>El Araby For Mechanical &amp; Electrical Supplies</t>
+          <t>Reda Aly</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>01142702406</t>
+          <t>01227236848</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>01142702406</t>
+          <t>01227236848</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>5 Gamea El Sisi St., Gharb El Sekka El Hadid, Manial shiha, Giza, Manial Shiha</t>
+          <t>Mohamed Mahmoud St., Imbaba, Giza, IMBABA</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>الميكانيكا</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1338,35 +1330,35 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/468184</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/360780</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Al Borg For General Services</t>
+          <t>Al Noaman</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>01068044346</t>
+          <t>01201403405</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>01068044346</t>
+          <t>01201403405</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Alex Matrouh Desert Rd., El alamein, North coast, EL ALAMEIN</t>
+          <t>8 El Adib Mohamed Zaitoun St., Semouha, Alexandria, SEMOUHA</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>أدوات النظافة</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1376,35 +1368,31 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/710162</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/469059</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Retaj Furniture</t>
+          <t>Tech Solution Of Egypt</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>01202877047</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>01202877047</t>
-        </is>
-      </c>
+          <t>0223619884</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>13 Ard El Maared St., Tanan Village, Qalyub, Kaliobeya, QALYUB</t>
+          <t>5 El Shawarby St. Off Kasr El Nil St., Downtown, Cairo, DOWNTOWN</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1414,35 +1402,35 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/519490</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/442596</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Expert For Computer</t>
+          <t>Of Design</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>01007313580</t>
+          <t>01281555626</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>01007313580</t>
+          <t>01281555626</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>18 Abou Bakr El Seddik St., Ezbet el nakhl, Cairo, EZBET EL NAKHL</t>
+          <t>17 El Batrawy St., Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1452,31 +1440,35 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/528068</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/462934</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>El Shroq Service Co.</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0228467264</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
+          <t>01098858585</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>01098858585</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>5014 Rd. 17, Mokattam, Cairo, MOKATTAM</t>
+          <t>El Gomhoureya St., El kalag, Kaliobeya, EL KALAG</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>أدوات النظافة</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1486,31 +1478,35 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/333744</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/417380</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Ragai Nassef For Restaurant Equipment</t>
+          <t>Art Group For Furniture</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0225121490</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr"/>
+          <t>01000905858</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>01000905858</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>13 El Mangala St., Darb Saada, El darb el ahmar, Cairo, EL DARB EL AHMAR</t>
+          <t>6 B El Fanneyeen El Askareen Bldgs. Youssef Abbas St., Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1520,31 +1516,35 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/687049</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/671780</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Magdy Abd Rabou Furniture</t>
+          <t>Computer House</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0242150496</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
+          <t>01000781384</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>01000781384</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>84 10th Of Ramadan St., Qalyub, Kaliobeya, QALYUB</t>
+          <t>5 El Sadat St., Kafr Berak El Khayyam, Kerdasa, Giza, Kerdasa</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1554,30 +1554,26 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/527225</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/556329</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>El Adel For Moving Furniture</t>
+          <t>El Bahnasy Furniture</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>01010038470</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>01010038470</t>
-        </is>
-      </c>
+          <t>0572240260</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>81 El Sabaq St., El Merryland, Heliopolis, Cairo, HELIOPOLIS</t>
+          <t>135 Aly Mosharrafa St., Damietta, Damietta, DAMIETTA</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1592,22 +1588,26 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/644835</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/503907</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Tech Me</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
+          <t>Yakout Tech For Computer</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>0233448610</t>
+        </is>
+      </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>26 El Nozha St., El Nozha, Heliopolis, Cairo, HELIOPOLIS</t>
+          <t>7, Sphinx Sq., Mohandeseen, Giza, MOHANDESEEN</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1622,35 +1622,35 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/683849</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/620238</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Milano Modern Furniture</t>
+          <t>El Lotus For Computer Supplies</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>01555548787</t>
+          <t>01275775566</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>01555548787</t>
+          <t>01275775566</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>El Mercato St., Umm el sid hill, Sharm el sheikh, UMM EL SID HILL</t>
+          <t>16 El Nasr St., El mansheya, Alexandria, EL MANSHEYA</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1660,35 +1660,35 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/703675</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/690875</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>United Arab Co. For Manufacturing Bakery Equipment</t>
+          <t>High Furniture</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>01288801163</t>
+          <t>01013936139</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>01288801163</t>
+          <t>01013936139</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Al Haganyeah Village, Damanhour, El beheira, Damanhour</t>
+          <t>26 El Thawra St., Almaza, Heliopolis, Cairo, HELIOPOLIS</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1698,35 +1698,35 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/480304</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/683159</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Arab Mechanical Engineers - AME</t>
+          <t>Mega For Computer Services</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>01277590084</t>
+          <t>01111154496</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>01277590084</t>
+          <t>01111154496</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Plot 314 El Tesaeen El Ganouby St., 5th Compound, New cairo, Cairo, NEW CAIRO</t>
+          <t>El Bahar El Ahmar St., El sherouk city, Cairo, EL SHEROUK CITY</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>الميكانيكا</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1736,31 +1736,35 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/626513</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/536822</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>El Ahram For Computer &amp; Systems</t>
+          <t>El Taweel Furniture</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0229242260</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
+          <t>01222975559</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>01222975559</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>122 Ramsis Tower, El Galaa St.  Ramsis Sq., Downtown, Cairo, DOWNTOWN</t>
+          <t>, Extension Of Makram Ebaid St., 8th District, Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1770,35 +1774,35 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/431834</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/307147</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Atlantis For Contracting</t>
+          <t>Kardouss Furniture</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>01022007739</t>
+          <t>01020002099</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>01022007739</t>
+          <t>01020002099</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Villa 66, Neighbourhood 27, 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
+          <t>51 Nabil El Waqqad St., Ard El Golf, Heliopolis, Cairo, HELIOPOLIS</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>الصحة والسلامة ومقاومة الحريق</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1808,30 +1812,26 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/656503</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/410071</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>I Technology</t>
+          <t>El Abd For Computer</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>01002884418</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>01002884418</t>
-        </is>
-      </c>
+          <t>0233264724</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>37 Abou Dawoud El Zahery St., 8th District, Nasr city, Cairo, NASR CITY</t>
+          <t>1 Saleh Mansour St.  Off Gamaet El Dewal El Arabeya St., Mohandeseen, Giza, MOHANDESEEN</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1846,30 +1846,30 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/699014</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/323070</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Legend International</t>
+          <t>Oscar Furniture</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>01012077999</t>
+          <t>01100121237</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>01012077999</t>
+          <t>01100121237</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Corniche El Nil St., Damietta, Damietta, DAMIETTA</t>
+          <t>21 Ahmed El Zomor St., Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1884,30 +1884,30 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/694021</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/707516</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Al Fares For Industrial Safety Supplies</t>
+          <t>New Age Co.</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>01110895856</t>
+          <t>01286973402</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>01110895856</t>
+          <t>01286973402</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>, Bldg. A, El Ordeneya, El Marwa Center, 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
+          <t>Km 26 Misr Alex Desert Rd., Abou rawash, Giza, ABOU RAWASH</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -1922,26 +1922,30 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/474142</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/697863</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Machines For Computer</t>
+          <t>Speed</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0227957232</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
+          <t>01002323137</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>01002323137</t>
+        </is>
+      </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>17 Aly Abdel Latif St., El sayeda zeinab, Cairo, EL SAYEDA ZEINAB</t>
+          <t>Sahl Hamza St., Off Haram St., El haram, Giza, EL HARAM</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1956,26 +1960,30 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/407100</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/503576</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Future Group</t>
+          <t>Star City For Computer</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0224555212</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr"/>
+          <t>01004073018</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>01004073018</t>
+        </is>
+      </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>7 El Sakhawy St., Roxy, Heliopolis, Cairo, HELIOPOLIS</t>
+          <t>26 Gamaet El Dewal El Arabeya St., Mohandeseen, Giza, MOHANDESEEN</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -1990,30 +1998,30 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/621180</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/383509</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Belal Furniture</t>
+          <t>El Mohandes</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>01223719155</t>
+          <t>01151475666</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>01223719155</t>
+          <t>01151475666</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>37 El Tahrir St., Saft El Laban, Boulak el dakrour, Giza, BOULAK EL DAKROUR</t>
+          <t>Ahmed Abd Rabou St., Shoubra el khaymah, Kaliobeya, SHOUBRA EL KHAYMAH</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2028,27 +2036,31 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/575943</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/410817</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Fawry Plus</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr"/>
+          <t>Ev Home &amp; Office Furniture</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>0236969311</t>
+        </is>
+      </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Abdel Moneim Riad St., El maragha, Sohag, EL MARAGHA</t>
+          <t>Plot 66, District 11Central Spine, 6th of october, Giza, 6th OF OCTOBER</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>الإلكترونيات</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2058,35 +2070,35 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/698304</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/469516</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Capital Plus</t>
+          <t>El Safa For Computer</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>01224781111</t>
+          <t>01156624949</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>01224781111</t>
+          <t>01156624949</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Shebin El Koum St., Downtown, Ismaileya, DOWNTOWN</t>
+          <t>3, Sphinx Sq., Mohandeseen, Giza, MOHANDESEEN</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>الصحة والسلامة ومقاومة الحريق</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2096,35 +2108,35 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/711173</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/620831</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Travel Maker Trips</t>
+          <t>Farouq Furniture</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>01286783479</t>
+          <t>01227562143</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>01286783479</t>
+          <t>01227562143</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2 Mohamed Ahmed St., Flat 303, Floor 3, Off Ahmed Badawy St., Shoubra, Cairo, SHOUBRA</t>
+          <t>18 El Hegaz St., El Amal City, Shoubra el khaymah, Kaliobeya, SHOUBRA EL KHAYMAH</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2134,22 +2146,30 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/625925</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/419883</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Carpiture Furniture</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
+          <t>Flair Office Furniture</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>01101003599</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>01101003599</t>
+        </is>
+      </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>El Shabab St., Obour city, Kaliobeya, OBOUR CITY</t>
+          <t>6 Salah El Din St., Zamalek, Cairo, ZAMALEK</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2164,30 +2184,30 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/645404</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/672650</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>El Alameya</t>
+          <t>El Nahda For Moving Furniture</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>01289226223</t>
+          <t>01030012007</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>01289226223</t>
+          <t>01030012007</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>5 Hussein Mohamed Ismail St., Faisal, Giza, FAISAL</t>
+          <t>Block 3 El Tayaran St.B, 7th District, Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2202,35 +2222,35 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/406263</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/520919</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>El Mola For Computer</t>
+          <t>Gamal Hafez Electronics</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>01148076867</t>
+          <t>01281814407</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>01148076867</t>
+          <t>01281814407</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>36 El Nil El Said St., El badrashin, Giza, EL BADRASHIN</t>
+          <t>205 Shoubra St., Shoubra, Cairo, SHOUBRA</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الإلكترونيات</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2240,22 +2260,26 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/611586</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/432035</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Home Centre</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr"/>
+          <t>Abdel Halim Sons Abou Samra Furniture</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>0222706365</t>
+        </is>
+      </c>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Omar Ibn El Khattab St., Nasr city, Cairo, NASR CITY</t>
+          <t>, Extension Of Makram Ebaid St., Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2270,7 +2294,1871 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/712557</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/600590</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Hesham Ayman For Computer Maintenance</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>01225552723</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>01225552723</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>24 Farouq El Sawy St., El Omraneya El Gharbeya, El haram, Giza, EL HARAM</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/493281</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Rocket For Electronic Marketing</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>01090761750</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>01090761750</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>El Narges Bldgs., Fatma El Sharbatly, 5th Compound, New cairo, Cairo, NEW CAIRO</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>الإلكترونيات</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/640695</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Tobaco Shop For Coffee Shop Supplies</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>01005610545</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>01005610545</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>1 Gamal Abdel Nasser St., Hadayek helwan, Cairo, HADAYEK HELWAN</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/644332</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Raqamyat</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>01050859295</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>01050859295</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>1 D/4 El Nasr St., New Maadi, Maadi, Cairo, MAADI</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>الإلكترونيات</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/688204</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Affandina Furniture</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>01002688423</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>01002688423</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>41 Ashra St., Warraq El Arab, El warak, Giza, EL WARAK</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/602062</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Classic Bed</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>01006893234</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>01006893234</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>97 Ahmed Orabi St., Ain shams, Cairo, AIN SHAMS</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/395061</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Cello Furniture</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>01557225582</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>01557225582</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>1 Abdel Hakim El Refaey St., Off Abbas El Akkad St., 8th District, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/671140</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Waw Designs</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>01223642847</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>01223642847</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>17 Rd . 263, Floor 1, Maadi, Cairo, MAADI</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/457697</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>El Anwar</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>01282307266</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>01282307266</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>6 Hassan El Anwar Sq., Misr el kadima, Cairo, MISR EL KADIMA</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/408508</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Foster</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>01122036797</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>01122036797</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>3 Umm El Moameneen St., Dar el salam, Cairo, DAR EL SALAM</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/456375</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>El Nouras</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>01286026019</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>01286026019</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>71 El Osra El Gadida Bldgs., Port fouad, Port said, PORT FOUAD</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/379905</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Nozom For Information Technology</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>01026865434</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>01026865434</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Villa 15, El Banafseg 2 District, 1st Compound, New cairo, Cairo, NEW CAIRO</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/705226</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>E-Busniess Solution Enabling Group - EBSEG</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>0227547580</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>8 A/3 Atef Khattab St.  Off Ahmed Kamel St., El Laselky Division, New Maadi, Maadi, Cairo, MAADI</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/453130</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Tech Village</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>01027052000</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>01027052000</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Villa 6 Qonsowa El Ghoury St., 1st Compound, New cairo, Cairo, NEW CAIRO</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/391359</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Nada Showroom</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>01289558191</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>01289558191</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Tanan Village, Qalyub, Kaliobeya, QALYUB</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/363465</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>El Khalil For Furniture</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>01151205555</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>01151205555</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>2 El Shorta St., El Fath City, Shoubra el khaymah, Kaliobeya, SHOUBRA EL KHAYMAH</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/476647</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Al Freeg For Engineering &amp; Trade</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>0238334376</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Central Spine, 12th District, 6th of october, Giza, 6th OF OCTOBER</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/346061</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Mix Station For Play Station</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>01000090047</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>01000090047</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>10 Ahmed Onsy St., Helwan, Cairo, HELWAN</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/642715</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Al Moataz Al Moriah Furniture</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>0226703234</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>, Extension Of Makram Ebaid St., 8th District, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/389053</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Golden Mind Software</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>01001982611</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>01001982611</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Sudan St., Mohandeseen, Giza, MOHANDESEEN</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/484918</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Egypt Print</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>01067670001</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>01067670001</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>18 El Bostan St., Bab el louk, Cairo, BAB EL LOUK</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/556152</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>El Bait El Said</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>01146573632</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>01146573632</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>El Marsad St., Helwan, Cairo, HELWAN</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/385701</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>A Data</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>01004025256</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>01004025256</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>4 El Adib Mohamed Zaitoun St., Semouha, Alexandria, SEMOUHA</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/468944</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Fire Extinguishers - Meteory</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>0226200068</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>81 Joseph Tito St., El nozha el gadida, Cairo, EL NOZHA EL GADIDA</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>الصحة والسلامة ومقاومة الحريق</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/468400</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Made In Egypt</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>01122286605</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>01122286605</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>35 Aly Ibn Abi Taleb St., Misr el kadima, Cairo, MISR EL KADIMA</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/673549</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>International For Hotel Services</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>01019190200</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>01019190200</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>14 West El Balad St., Abou rawash, Giza, ABOU RAWASH</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/475142</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Madar Home Signature</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>01068841164</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>01068841164</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Mohamed Naguib Spine, North Investors, New cairo, Cairo, NEW CAIRO</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/692473</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>El Forsan For Cleaning Tools</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>01005092890</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>01005092890</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>, Central Spine, Lailat El Qadr Sq., 12th District, 6th of october, Giza, 6th OF OCTOBER</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>أدوات النظافة</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/651393</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Sky For Control Boards</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>01061919986</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>01061919986</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Mohamed Hafez St., El Ordoneya, 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/620601</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Mansour Furniture</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>01223593125</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>01223593125</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>93 A Gesr El Suez St., Heliopolis, Cairo, HELIOPOLIS</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/423160</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>01009635681</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>01009635681</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>, Extension Of El Gomhoureya St., El shark district, Port said, EL SHARK DISTRICT</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/315753</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>El Shehab Group For Computer</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>01221457057</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>01221457057</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>19 Mohamed Abdel Salam St., El khosous, Kaliobeya, EL KHOSOUS</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/499665</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Marvel Integrated Solutions</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>01005311730</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>01005311730</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>21 Nagaty Serag St., 8th Zone, 8th District, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/687285</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Eid For Cars Electricity</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>01220816301</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>01220816301</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Commercial Market St., Saqiet Mekky, Giza, Giza, GIZA</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/432300</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Techical Workshop For Furniture Painting</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>01016081742</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>01016081742</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>13 Aly Mahmoud El Essawy St., El Gezirah, Dar el salam, Cairo, DAR EL SALAM</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/498823</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Future For Computer</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>01114005182</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>01114005182</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>, 5th Neighbourhood, 1St District, El Sheikh Zayed, 6th of october, Giza, 6th OF OCTOBER</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/471075</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Forbed</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr"/>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>155 El Teraa El Boulaqeya St., Shoubra, Cairo, SHOUBRA</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/432624</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>White Horse</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>01009916682</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>01009916682</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>64 Mohamed Farid St., El Montazah, Sidi beshr kebly, Alexandria, SIDI BESHR KEBLY</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/599552</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Master For Furniture</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>01024623453</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>01024623453</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>29 Mohamed Kamel El Harouny St., Off Ahmed Fakhry St., 6th Zone, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/386670</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Golden Eyes</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>01005307279</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>01005307279</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Omar Ibn Abdel Aziz St., Abou zaabal, Kaliobeya, ABOU ZAABAL</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/345102</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Ibs - International Business Systems</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>01004193882</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>01004193882</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>7 Mohamed Said St., El Sefarat District, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/446908</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Majestic Home Furniture</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>0226213145</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>81 Joseph Tito St.,  Off Rd. Sindbad, El nozha el gadida, Cairo, EL NOZHA EL GADIDA</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/382038</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Tabarak Center</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>01004849110</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>01004849110</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>El Eshreen St., Ain shams el sharkeya, Cairo, AIN SHAMS EL SHARKEYA</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/318451</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>El Domiateya For Furniture</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>01008038053</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>01008038053</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>1 Ahmed Zeyada St., El marg, Cairo, EL MARG</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/562618</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Mattar Information Technology - MIT</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>01000515160</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>01000515160</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>3 El Sheikh Hamza Fath Allah St.  Off Misr &amp; Sudan St., Hadayek el kobba, Cairo, HADAYEK EL KOBBA</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/581994</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr"/>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>14 El Marwa Towers Ahmed Tayseer St., Ard El Golf, Heliopolis, Cairo, HELIOPOLIS</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>الإلكترونيات</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/578592</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Compu House</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>01062201515</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>01062201515</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>13 Dar El Salam St., Hamamat el kobba, Cairo, HAMAMAT EL KOBBA</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/401382</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Linkit For Software</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>01066380809</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>01066380809</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Plot 168Central Zone, New damietta, Damietta, NEW DAMIETTA</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/632173</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Zika Store For Computer</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>01000121415</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>01000121415</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>1 Masged Bayoumi Moqbel St., Imbaba, Giza, IMBABA</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/574723</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Mahgoub Sons</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>01118435590</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>01118435590</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Mohamed Abdel Daem St., Mansheyet El Bakkary, Faisal, Giza, FAISAL</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/381232</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve starting scraper by automatically stopping if already running
Modify the `doStart` function to gracefully stop any existing scraper process before initiating a new one, preventing "already running" errors.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 2a1fad78-d05e-42f0-ad61-6fa4ea0cba54
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 8f3fd443-1d50-45f8-be4b-9dc1299b2fd2
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/0ea4e3a5-1e4e-40d5-826b-5b1dabac3eb2/2a1fad78-d05e-42f0-ad61-6fa4ea0cba54/A0TXRhK
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backup_temp.xlsx
+++ b/backup_temp.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2290,6 +2290,1834 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Forbed</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Bank Misr St., Garas Sons Bldg., Mallawi, El menia, MALLAWI</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/713276</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Almsrya Furniture</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>01013008585</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>01013008585</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>, 5th Zone, Sadat city, El monofeya, SADAT City</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/687542</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Technological Development Center - Education Directorate - El Daqahleya</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>0502381907</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Gamaet El Dewal El Arabeya St.  Off Port Said St., El mansoura, El dakahleya, EL MANSOURA</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/360775</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Dynamics Link</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>0220800759</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>26 Aly Amin St., Extension Of Mostafa El Nahhas St., 1st Zone, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/543536</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>EgyComm</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>01119793013</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>01119793013</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>186 Port Said St., Sporting, Alexandria, SPORTING</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/711547</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>X Game Stores</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>01000138959</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>01000138959</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Km 52 Misr Ismaileya Desert Rd., 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/669320</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>El Hamd</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>01007984131</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>01007984131</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>saad zaghloul st., Zefta, El gharbeya, ZEFTA</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/336469</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Smart Network</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>01111501387</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>01111501387</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Atteya El Sawalhy St.  Extension Of Makram Ebaid St., El Serag City Mall Towers, Entrance B, Floor 2, 8th District, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/564303</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>El Zahabeya For Computers</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>0623193319</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>El Khedr St., Floor 1, El ghareeb, Suez, EL GHAREEB</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/471017</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>IT Planet</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>01113331172</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>01113331172</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>3 El Obour Bldgs. Salah Salem Rd., Flat 2, Floor 16, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/687793</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Khalifa Trade</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>0552320533</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>22 El Galaa St., El zagazig, El sharkeya, EL ZAGAZIG</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/328961</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Wood &amp; Plexi</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>01006170270</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>01006170270</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>81 El Dobbat Bldgs. Rd. 22, Mostafa kamel, Alexandria, MOSTAFA KAMEL</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/712967</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Shoppers Technologies</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>035467702</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>1 Mostafa Kamel St., Off El Horreya Rd., Roushdy, Alexandria, ROUSHDY</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/606306</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>El Masreya</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>01006152091</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>01006152091</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Gamea El Sahly St., Kafr el zayat, El gharbeya, KAFR EL ZAYAT</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/342418</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Forbed</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>El Mostashfa St., Gerga, Sohag, GERGA</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/713289</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Ava Tech Smart Solutions</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>01557735939</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>01557735939</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>3 El Khamraweya St., El Batal Tower, Shoubra, Cairo, SHOUBRA</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/661698</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Qassed Karim</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>01114753224</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>01114753224</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>77 El Mansheya St., El Tawabeq, Faisal, Giza, FAISAL</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/332763</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>El Safwa Furniture</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>01018497999</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>01018497999</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>7 El Delta St., Shebein el kanater, Kaliobeya, SHEBEIN EL KANATER</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/517588</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Friend Computer System</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>01129646435</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>01129646435</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>16 Abdel Hamid El Sayed St., Dar el salam, Cairo, DAR EL SALAM</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/456363</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Bedir Recliner And Furniture</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>01112880033</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>01112880033</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>42 Naguib Mahfouz St., 8th District, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/710910</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Smart Wood</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>01120060872</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>01120060872</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>4 Sekket El Nazir St., El moneeb, Giza, EL MONEEB</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/617380</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Topsession</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>01009422887</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>01009422887</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>20 El Shity St.  Off El Bahr St., Floor 2, Tanta, El gharbeya, TANTA</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/458973</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>El Fouly Showroom</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>01223470727</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>01223470727</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>22 El Mohawelat St., El Talbeya, El haram, Giza, EL HARAM</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/416086</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Malak Rouhy For Furniture</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>01225477621</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>01225477621</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>25 Masged Namera St., Hadayek El Maadi, Maadi, Cairo, MAADI</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/684562</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>El Masria For Computers</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>01280006650</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>01280006650</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Television St., LUXOR, Luxor, Luxor, Luxor</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/458683</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Horus For Computer Services</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>01225908071</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>01225908071</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>13 Abdel Sattar El Attar St., Banha, Kaliobeya, BANHA</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/521485</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Forbed</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>El Sheikh Mohamed Abdou St., El ghareeb, Suez, EL GHAREEB</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/713469</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>El Hamd Showroom</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>01159259277</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>01159259277</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>156 Ahmed Orabi St., Shoubra el khaymah, Kaliobeya, SHOUBRA EL KHAYMAH</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/410542</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>B.TECH</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Plot 45, Central Zone, New damietta, Damietta, NEW DAMIETTA</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/651821</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>A2M</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>01009535966</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>01009535966</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>200 Sudan St., Mohandeseen, Giza, MOHANDESEEN</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/379922</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Saher Shop For Computer</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>01112901976</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>01112901976</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>1 Abou Setta St.  Off Hassan Youssef St., El Sheddeya, Banha, Kaliobeya, BANHA</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/522055</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>El Nagdy</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>0553500889</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>el noqrashy st., Abou kebeir, El sharkeya, ABOU KEBEIR</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/329681</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>King Office Furniture</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>035235512</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>79 Sidi Gaber El Sheikh Ali El Teram St., Sidi gaber el sheikh, Alexandria, SIDI GABER EL SHEIKH</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/522539</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Yassin</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>01068322157</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>01068322157</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>22 Ain Shams St., Helmeyet el zaitoun, Cairo, HELMEYET EL ZAITOUN</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/322091</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Nile Home</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>01202705833</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>01202705833</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>, Central Spine, 10th District, 6th of october, Giza, 6th OF OCTOBER</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/613194</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Elhandasya Khalid Ezz El Din For Hotel &amp; Restaurant supply</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>01009333013</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>01009333013</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>12 El Madars St.  El Remaya Sq., Faisal, Giza, FAISAL</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/584284</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>El Safwa For Office Furniture</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>01206112532</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>01206112532</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>El Mizana , Plaza Tower, Kafr el dawar, El beheira, KAFR EL DAWAR</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/635782</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>I Station</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>01001799743</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>01001799743</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>El Khamseen St., Zahraa El Maadi, Maadi, Cairo, MAADI</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/637598</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>El Khayyat</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>01115980600</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>01115980600</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>El Masanea St., Abou zaabal, Kaliobeya, ABOU ZAABAL</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/421329</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Magic Group</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>0237805388</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>4 El Farouq St., El Tawabeq, Faisal, Giza, FAISAL</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/427828</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>El Farouq For Electricity Equipment Showroom</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>01115127047</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>01115127047</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>16 El Moatasem Bellah St.  Off El Tahrir St., Saft El Labn, Boulak el dakrour, Giza, BOULAK EL DAKROUR</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/576459</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Effective Solutions</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>01226933342</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>01226933342</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Plot 140, , Badr city, Cairo, BADR CITY</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/581052</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Emad Showroom</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>01001178135</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>01001178135</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>El Gharby St., Helwan, Cairo, HELWAN</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/385949</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>01225455093</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>01225455093</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>El Safa &amp; El Marwa St., Faisal, Giza, FAISAL</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/406464</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>El Aseel Furniture</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>01007569650</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>01007569650</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>3 El Mathan St., El Sayala, Damietta, Damietta, DAMIETTA</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/509567</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Egypt Laptop</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>01099472998</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>01099472998</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>5 Rd. 311, Off Mostafa Kamel St., Semouha, Alexandria, SEMOUHA</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/469058</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>No Name Furniture</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>01004780139</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>01004780139</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>5 Hussein Sherin St., Loran, Alexandria, LORAN</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/470367</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Engaz Shop</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>0472555979</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>3 El Sharekat St.Qortoba Tower,  floor 3, Disuq, Kafr el sheikh, DISUQ</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/620745</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Nour El Hoda For Furniture Moving</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>01272187545</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>01272187545</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>114 El Guish St., Bab el shaareya, Cairo, BAB EL SHAAREYA</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/675725</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Smart Net Serv</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>0224029442</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>4 El Obour Bldgs., Salah Salem Rd., Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/436442</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Make starting and stopping the scraper more reliable
Switch the dashboard's start and stop functionality from WebSocket to HTTP requests to improve reliability and responsiveness.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 2a1fad78-d05e-42f0-ad61-6fa4ea0cba54
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 7d417d23-70e5-4c07-8dfd-2567831c2412
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/0ea4e3a5-1e4e-40d5-826b-5b1dabac3eb2/2a1fad78-d05e-42f0-ad61-6fa4ea0cba54/JYJXN5n
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backup_temp.xlsx
+++ b/backup_temp.xlsx
@@ -461,28 +461,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Multi Tech</t>
+          <t>El Badry Showroom</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>01005544455</t>
+          <t>01224043101</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>01005544455</t>
+          <t>01224043101</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2 Ramo Bldgs., El Motamayez District, 6th of october, Giza, 6th OF OCTOBER</t>
+          <t>2 Fouad Emam St., Shoubra el khaymah, Kaliobeya, SHOUBRA EL KHAYMAH</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -492,35 +492,35 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/689385</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/418648</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Farag Abdel Khaleq For Electronics</t>
+          <t>El Basel For Furniture</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>01008731190</t>
+          <t>01112422626</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>01008731190</t>
+          <t>01112422626</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Block 19, Ain Shams Bldgs., Ain shams, Cairo, AIN SHAMS</t>
+          <t>23 El Bosta St., Geziret Mohamed Village, El warak, Giza, EL WARAK</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>الإلكترونيات</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -530,35 +530,35 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/336031</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/599762</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>International Co. For Computers</t>
+          <t>Target For Import And Export</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>01004567281</t>
+          <t>01110444615</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>01004567281</t>
+          <t>01110444615</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Abdel Moneim Riad St., Kafr shoukr, Kaliobeya, KAFR SHOUKR</t>
+          <t>, 1St Industrial Zone, El katameya, Cairo, EL KATAMEYA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -568,35 +568,35 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/311092</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/685213</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>The Specialized Co. For Goods &amp; Furniture Transport</t>
+          <t>Power System For Computer</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>01060110710</t>
+          <t>01289601448</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>01060110710</t>
+          <t>01289601448</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>21 El Guish St., Ataba, Cairo, ATABA</t>
+          <t>Mostafa El Araby St., El Koum El Akhdar, Faisal, Giza, FAISAL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -606,35 +606,35 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/501720</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/424157</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Server For Computer</t>
+          <t>El Hamd Service Center For Electronics &amp; Maintenance</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01149929397</t>
+          <t>01224834563</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>01149929397</t>
+          <t>01224834563</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>21 Amin Hamada St., Ezbet el nakhl, Cairo, EZBET EL NAKHL</t>
+          <t>Rd. 1, Ghebrial, Alexandria, GHEBRIAL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الإلكترونيات</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -644,35 +644,35 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/522442</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/392217</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Abnaa Tanta For Cars Electricity</t>
+          <t>Ebay</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>01144530111</t>
+          <t>01007110210</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>01144530111</t>
+          <t>01007110210</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>28 Ain Shams St., Ain shams, Cairo, AIN SHAMS</t>
+          <t>23 Ramsis St., El Korba, Heliopolis, Cairo, HELIOPOLIS</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>الكهرباء والكابلات والأسلاك</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -682,30 +682,30 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/477182</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/420237</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>IT Systematic</t>
+          <t>El Masa</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>01090718730</t>
+          <t>01004994626</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>01090718730</t>
+          <t>01004994626</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>, 10th Neighbourhood, 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
+          <t>Selim St., Koum Bakkar, Faisal, Giza, FAISAL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -720,35 +720,35 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/651615</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/380508</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Railways Co. For Integrated Services</t>
+          <t>3M For Computer</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>01126086249</t>
+          <t>01140336393</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>01126086249</t>
+          <t>01140336393</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Saad Zaghloul St.  El Mahatta Sq., Downtown, Aswan, DOWNTOWN</t>
+          <t>31 Gamal Abdel Nasser St. Farid Zaky Division, Hadayek helwan, Cairo, HADAYEK HELWAN</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>أدوات النظافة</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -758,35 +758,35 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/534964</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/445117</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Egyemb Electronics</t>
+          <t>Ebtakarna Lak</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>01009735581</t>
+          <t>01000679000</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>01009735581</t>
+          <t>01000679000</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>El Gamea Alley, Bein el sarayat, Giza, BEIN EL SARAYAT</t>
+          <t>11 Palestine St., Off El Laselky St., Palestine Sq., New Maadi, Maadi, Cairo, MAADI</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>الإلكترونيات</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -796,35 +796,35 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/506846</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/616496</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Egyptian Group For Computers</t>
+          <t>Saloni</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>01229808254</t>
+          <t>01000255880</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>01229808254</t>
+          <t>01000255880</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>162 Haram St., El Arish, El haram, Giza, EL HARAM</t>
+          <t>, Customer Service, Heliopolis, Cairo, HELIOPOLIS</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -834,35 +834,35 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/394112</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/425328</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Idea Industry Furniture</t>
+          <t>Alam El Computer Center</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>01090707279</t>
+          <t>01001808539</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>01090707279</t>
+          <t>01001808539</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2 El Khamseen St. Off Sayed Abou Damaah St., El nozha el gadida, Cairo, EL NOZHA EL GADIDA</t>
+          <t>9 Mahmoud Aref St, Off El Shishiny St., Faisal, Giza, FAISAL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -872,31 +872,35 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/515218</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/672789</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>El Mallwany Home Décor Mall</t>
+          <t>Time Computer</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>034872221</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>01288111293</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>01288111293</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>20 El Hamamil St., El mansheya, Alexandria, EL MANSHEYA</t>
+          <t>Eid Khairullah St., Agami, Alexandria, AGAMI</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -906,30 +910,30 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/351805</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/708464</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ghost For Computer Maintenance</t>
+          <t>Shaqawa</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>01124402004</t>
+          <t>01004000146</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>01124402004</t>
+          <t>01004000146</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14 Abou Zaid Farag St. Off El Matarawy St., El matareya, Cairo, EL MATAREYA</t>
+          <t>34 Awlad Ouf St., El Talbeya, El haram, Giza, EL HARAM</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -944,31 +948,35 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/460195</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/323509</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>El Batal Showroom</t>
+          <t>Sama For Computer</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0226975225</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>01006965973</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>01006965973</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14 Ibrahim Tantawy St., El herafeyeen, Cairo, EL HERAFEYEEN</t>
+          <t>28 El Gadid St., Kerdasa, Giza, Kerdasa</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -978,35 +986,35 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/549147</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/558230</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Gamalco Furniture</t>
+          <t>El Tawhid For Computer</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>01112517974</t>
+          <t>01112853956</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>01112517974</t>
+          <t>01112853956</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>160 Faisal St., El Koum El Akhdar, Faisal, Giza, FAISAL</t>
+          <t>70 Ain Shams St., Ain shams el sharkeya, Cairo, AIN SHAMS EL SHARKEYA</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1016,35 +1024,35 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/510890</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/377324</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sodcks</t>
+          <t>Smart Idea</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>01003035696</t>
+          <t>01285266341</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>01003035696</t>
+          <t>01285266341</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>4 El Mohemat Bldgs., Emtedad Ramsis St., Nasr city, Cairo, NASR CITY</t>
+          <t>7 Amin El Leithy St., Amer City, Boulak el dakrour, Giza, BOULAK EL DAKROUR</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>الصحة والسلامة ومقاومة الحريق</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1054,30 +1062,22 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/526534</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/447240</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TA Group</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>01275033988</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>01275033988</t>
-        </is>
-      </c>
+          <t>Mazloum Home</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>50 A Mohamed Mazhar St., Zamalek, Cairo, ZAMALEK</t>
+          <t>1 Mohamed Taimour St., Saint Fatima, Heliopolis, Cairo, HELIOPOLIS</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1092,35 +1092,35 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/458467</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/443149</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>New Power For Electrical Supplies And Metal Sheets</t>
+          <t>Nour Steel For Restaurant And Hotel Equipment Supplies</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>01060313293</t>
+          <t>01222252311</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>01060313293</t>
+          <t>01222252311</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>53 El Husseiny Bldg. Naguib El Rihany St., Floor 7, Downtown, Cairo, DOWNTOWN</t>
+          <t>Green Towers - Tower 6, Semouha, Alexandria, SEMOUHA</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>الكهرباء والكابلات والأسلاك</t>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1130,27 +1130,35 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/698861</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/688235</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Aman</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
+          <t>El Madina Furniture</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>01003933036</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>01003933036</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>El Eman St., Agami, Alexandria, AGAMI</t>
+          <t>38 Abbas Anany St., El badrashin, Giza, EL BADRASHIN</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>الإلكترونيات</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1160,35 +1168,35 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/698097</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/606380</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MA Showroom</t>
+          <t>El Walid For Computer</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>01090682462</t>
+          <t>01099331470</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>01090682462</t>
+          <t>01099331470</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>El Gawazat St., Kafr sakr, El sharkeya, KAFR SAKR</t>
+          <t>7 Madraset El Motafaweqin St., Ain shams, Cairo, AIN SHAMS</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1198,35 +1206,35 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/351555</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/304663</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Jasmine Establishment For Trade &amp; Electromechanical Contracting</t>
+          <t>El Boraie For Coffee Shop Supplies</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>01550490092</t>
+          <t>01004358301</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>01550490092</t>
+          <t>01004358301</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>50 Abdel Salam Mabrouk St., El sharabeya, Cairo, EL SHARABEYA</t>
+          <t>8 Abou El Magd Abou Rehab St., Hadayek El Maadi, Maadi, Cairo, MAADI</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>الصحة والسلامة ومقاومة الحريق</t>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1236,35 +1244,35 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/613851</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/684571</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Choice Interiors</t>
+          <t>RKB Plast</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>01030831899</t>
+          <t>01224499742</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>01030831899</t>
+          <t>01224499742</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>73 Abou Dawoud El Zahery St., Off Makram Ebaid St., Nasr city, Cairo, NASR CITY</t>
+          <t>, Plastic Industrey Complex - Unit 17- 80, Mirghem, Alexandria, MIRGHEM</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1274,35 +1282,35 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/669966</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/690445</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>El Gezirah For Computer</t>
+          <t>Abdou For Electronics Maintenance</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>01223326255</t>
+          <t>01098912380</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>01223326255</t>
+          <t>01098912380</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>62 El Orouba St., Warraq El Arab, El warak, Giza, EL WARAK</t>
+          <t>29 Rd. 10, Zahraa Ain Shams, Ain shams el sharkeya, Cairo, AIN SHAMS EL SHARKEYA</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الإلكترونيات</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1312,31 +1320,35 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/594884</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/653239</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Kasr El Houda Furniture</t>
+          <t>Al Mohtaseb Software</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0226525932</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr"/>
+          <t>01024226678</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>01024226678</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>24 Shagaret Mariam St., El matareya, Cairo, EL MATAREYA</t>
+          <t>1 El Sheikh Mohamed El Nady St., Off Makram Ebaid St., 6th Zone, Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1346,30 +1358,30 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/460357</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/423840</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Spark Egypt For Trading</t>
+          <t>Matrix For Computer Services</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>01090777876</t>
+          <t>01225661048</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>01090777876</t>
+          <t>01225661048</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>8 B Youssef Abas St., Nasr city, Cairo, NASR CITY</t>
+          <t>2 Othman Ibn Affan St., Kebaa city, Cairo, KEBAA CITY</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1384,30 +1396,30 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/629281</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/481671</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Mega Mix For Computer</t>
+          <t>El Hagry For Computer</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>01006867734</t>
+          <t>01126534898</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>01006867734</t>
+          <t>01126534898</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2 El Abasiry St., El moneeb, Giza, EL MONEEB</t>
+          <t>34 Dayer El Nahya St., Geziret Mohamed Village, El warak, Giza, EL WARAK</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1422,30 +1434,26 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/655575</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/599727</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Friends For Computer Services</t>
+          <t>High New Cairo Institute For Administrative Sciences &amp; Computer</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>01064040542</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>01064040542</t>
-        </is>
-      </c>
+          <t>0222461112</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>126 Mostafa El Nahhas St., 6th Zone, Nasr city, Cairo, NASR CITY</t>
+          <t>7th Neighbourhood, 1st Compound, New cairo, Cairo, NEW CAIRO</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1460,30 +1468,30 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/596679</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/425132</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Edu Vision For Educational Supplies</t>
+          <t>El Mokhtar Furniture</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>01063584444</t>
+          <t>01125923251</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>01063584444</t>
+          <t>01125923251</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Villa 37, El Sheikh Zayed, 6th of october, Giza, 6th OF OCTOBER</t>
+          <t>125 El Gesr El Barrany St.  El Matbaa Sq., Dar el salam, Cairo, DAR EL SALAM</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1498,22 +1506,30 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/460140</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/507234</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Tech Me</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
+          <t>VIP For Computer Services</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>01013799204</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>01013799204</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>114 26th Of July St., Zamalek, Cairo, ZAMALEK</t>
+          <t>34 Abbas El Akkad St., Geziret el dahab, Giza, GEZIRET EL DAHAB</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1528,35 +1544,35 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/683842</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/502498</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Bedir Recliner And Furniture</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>01112880033</t>
+          <t>01005055230</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>01112880033</t>
+          <t>01005055230</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>24 Tut Ankh Amoun St., Semouha, Alexandria, SEMOUHA</t>
+          <t>41 Nasr Nassar St., Ard El Haddad, Imbaba, Giza, IMBABA</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1566,26 +1582,30 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/710911</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/353857</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mina Art</t>
+          <t>Stivan Furniture</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0244474585</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr"/>
+          <t>01010183939</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>01010183939</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>El Qanater El Khaireya Rd., Basoos, Kaliobeya, BASOOS</t>
+          <t>, Service Spine, 11th District, 6th of october, Giza, 6th OF OCTOBER</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1600,26 +1620,22 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/306304</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/668164</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ITS - Integrated Technology Services</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>0227547147</t>
-        </is>
-      </c>
+          <t>E-Planet For Educational Services</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>6 A2 Sayed Nada St.  El Laselky Division, New Maadi, Maadi, Cairo, MAADI</t>
+          <t>Sabry El Bekbashy St., Downtown, El fayoum, DOWNTOWN</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1634,31 +1650,31 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/451067</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/692021</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Misr International For Electromechanical Works</t>
+          <t>Be Smart Solution</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0237812798</t>
+          <t>035492386</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>5 Ahmed Seddik St., Off Hassan Metwally St., El haram, Giza, EL HARAM</t>
+          <t>2 El Mahdy St., Miami, Alexandria, MIAMI</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>الميكانيكا</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1668,35 +1684,35 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/689582</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/617353</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Elmanasrah</t>
+          <t>Shahd &amp; Fady</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>01064494524</t>
+          <t>01004009114</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>01064494524</t>
+          <t>01004009114</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>, El Manasra, Giza, Giza, GIZA</t>
+          <t>El Shaheed Anwar St., El baragil, Giza, EL BARAGIL</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1706,35 +1722,31 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/685475</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/348852</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Robabekya Furniture</t>
+          <t>Global IT</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>01025274802</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>01025274802</t>
-        </is>
-      </c>
+          <t>0233807934</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>, 2nd Neighbourhood, 1St District, El Sheikh Zayed, 6th of october, Giza, 6th OF OCTOBER</t>
+          <t>76 Ahmed El Zayyat St., Dokki, Giza, DOKKI</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1744,31 +1756,35 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/600021</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/671362</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>It Queue</t>
+          <t>Collection For Furniture</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0223493345</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
+          <t>01100315004</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>01100315004</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>5 A Hafez Ramadan St.  Off Makram Ebaid St., 6th Zone, Nasr city, Cairo, NASR CITY</t>
+          <t>El Horreya St., Ezbet Khairallah, Dar el salam, Cairo, DAR EL SALAM</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1778,30 +1794,30 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/599128</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/649260</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Next End</t>
+          <t>Compu Lap Technology</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>01007800727</t>
+          <t>01007905808</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>01007800727</t>
+          <t>01007905808</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1 El Nasr st., Floor 3, Off Salem Khiza St., El Amal City, Imbaba, Giza, IMBABA</t>
+          <t>136 El Hegaz St., Heliopolis, Cairo, HELIOPOLIS</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1816,31 +1832,31 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/630036</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/426103</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>El Hamd Showroom</t>
+          <t>Soft Computer Services</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0132522751</t>
+          <t>0653446555</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Abdel Moneim Riad St., Kafr shoukr, Kaliobeya, KAFR SHOUKR</t>
+          <t>El Central El Seyahy St.  Off Sheraton Rd., Sekala, Hurghada, SEKALA</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1850,35 +1866,35 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/311265</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/393763</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>El Alamia For Engineering And Electrical Panels Manufacturing</t>
+          <t>El Sharqawy Mall</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>01003633325</t>
+          <t>01221484651</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>01003633325</t>
+          <t>01221484651</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>9 El Sheikh Aly Mahmoud St., Floor 4, El Mahkama Square, Heliopolis, Cairo, HELIOPOLIS</t>
+          <t>El Galaa St., Quwasnah, El monofeya, QUWASNAH</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>الكهرباء والكابلات والأسلاك</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1888,35 +1904,31 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/502993</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/314343</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Epsilon Egypt For Powder Coating &amp; Metal Processing</t>
+          <t>Wizard For Computer Maintenance</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>01007145945</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>01007145945</t>
-        </is>
-      </c>
+          <t>035936026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Plot 69 &amp; 70250 Feddan Industrial Area, Badr city, Cairo, BADR CITY</t>
+          <t>26 Adonis St., El ibrahimeya, Alexandria, EL IBRAHIMEYA</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>الصحة والسلامة ومقاومة الحريق</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1926,35 +1938,35 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/466495</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/473371</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>El Rawda For Computer</t>
+          <t>El Hamd For Office Furniture</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>01144685582</t>
+          <t>01095921098</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>01144685582</t>
+          <t>01095921098</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>18 El Bostan St., Bab el louk, Cairo, BAB EL LOUK</t>
+          <t>Kobry El Adweya, El salam city, Cairo, EL SALAM CITY</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1964,31 +1976,31 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/556104</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/475708</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Tami Systems</t>
+          <t>Sobol Engineering Design Solutions</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0224724737</t>
+          <t>0221913371</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>44 A , El Swesry District, Nasr city, Cairo, NASR CITY</t>
+          <t>18 El Wehda El Arabeya St., Floor 2, Gesr el suez, Cairo, GESR EL SUEZ</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الميكانيكا</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1998,30 +2010,30 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/310860</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/539813</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Kiwan Furniture</t>
+          <t>El Adawy For Furniture</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>01002963030</t>
+          <t>01112643615</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>01002963030</t>
+          <t>01112643615</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>6 El Sayala St., El Sayala, Damietta, Damietta, DAMIETTA</t>
+          <t>abdel samea el haddad st., El Omraneya El Gharbeya, El haram, Giza, EL HARAM</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2036,30 +2048,30 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/510714</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/314783</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>El Forsan  For Moving Furniture</t>
+          <t>Concept For Furniture</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>01212495984</t>
+          <t>01149360436</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>01212495984</t>
+          <t>01149360436</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Gamila Bouhraid, El seyouf, Alexandria, EL SEYOUF</t>
+          <t>Plot 56, 1st District Services Zone, 5th Compound, New cairo, Cairo, NEW CAIRO</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2074,35 +2086,35 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/633169</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/665389</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Elwan Group For Galvanized Wires</t>
+          <t>Samer Shekhani For Restaurants Equipment</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>01127512960</t>
+          <t>01112176687</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>01127512960</t>
+          <t>01112176687</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>, Corniche Kafr Hegazy, El mahalla el kobra, El gharbeya, EL MAHALLA EL KOBRA</t>
+          <t>, El Hosary Sq., Central Spine, Alaa El Din Towers, Tower A, 7th District, 6th of october, Giza, 6th OF OCTOBER</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>الكهرباء والكابلات والأسلاك</t>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2112,31 +2124,35 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/695802</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/644892</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>El Nil For General Supplies</t>
+          <t>El Khalil</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0554365999</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr"/>
+          <t>01004552797</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>01004552797</t>
+        </is>
+      </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>, El Ordoneya, 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
+          <t>Port Said St., As-santah, El gharbeya, AS-SANTAH</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>الصحة والسلامة ومقاومة الحريق</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2146,35 +2162,35 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/633514</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/349907</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Abou Ahmed For Furniture Painting</t>
+          <t>Technowow</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>01008760525</t>
+          <t>01013388535</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>01008760525</t>
+          <t>01013388535</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>9 Masged El Saleheen St., Bashtil Village, Auseem, Giza, AUSEEM</t>
+          <t>, Hadaeq October, Small Industries Compound, Bldg. 4, 6th of october, Giza, 6th OF OCTOBER</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2184,35 +2200,31 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/540924</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/575148</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>El Masry Furniture</t>
+          <t>Rayan Net Fom Computer</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>01100315119</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>01100315119</t>
-        </is>
-      </c>
+          <t>0238321196</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>27 Abdel Hamid El Deeb St., Shoubra, Cairo, SHOUBRA</t>
+          <t>., 11th District, 6th of october, Giza, 6th OF OCTOBER</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2222,35 +2234,27 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/433838</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/438046</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Hany Aly For Computer Services</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>01151799285</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>01151799285</t>
-        </is>
-      </c>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>36 El Matbaa St., Floor 1, El Matbaa, Faisal, Giza, FAISAL</t>
+          <t>Gamal Abdel Nasser St., Nasser, Benisuef, Nasser</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الإلكترونيات</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2260,35 +2264,35 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/581287</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/698560</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Vigour Unity</t>
+          <t>Eyelets For Software</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>01210389067</t>
+          <t>01009996430</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>01210389067</t>
+          <t>01009996430</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>14 El Hegaz St., Hegaz Square, Heliopolis, Cairo, HELIOPOLIS</t>
+          <t>97 Khofo St.  Off Haram St., El haram, Giza, EL HARAM</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>الكهرباء والكابلات والأسلاك</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2298,7 +2302,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/693315</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/540602</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update scraper controls to use POST requests
Modify API endpoints from GET to POST for starting and stopping the scraper, and update the dashboard to reflect these changes.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 2a1fad78-d05e-42f0-ad61-6fa4ea0cba54
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: ad19ea92-ce17-44d9-a35d-a8a55e99c06a
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/0ea4e3a5-1e4e-40d5-826b-5b1dabac3eb2/2a1fad78-d05e-42f0-ad61-6fa4ea0cba54/ozuI7Oa
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backup_temp.xlsx
+++ b/backup_temp.xlsx
@@ -461,23 +461,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>El Badry Showroom</t>
+          <t>Hamis Fine Art</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>01224043101</t>
+          <t>01090013024</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>01224043101</t>
+          <t>01090013024</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2 Fouad Emam St., Shoubra el khaymah, Kaliobeya, SHOUBRA EL KHAYMAH</t>
+          <t>12 Abou Bakr El Seddik St., El Mariouteya, Faisal, Giza, FAISAL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -492,35 +492,35 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/418648</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/454972</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>El Basel For Furniture</t>
+          <t>MG For Engineering &amp; Electronic Industries</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>01112422626</t>
+          <t>01225331212</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>01112422626</t>
+          <t>01225331212</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>23 El Bosta St., Geziret Mohamed Village, El warak, Giza, EL WARAK</t>
+          <t>1 Shonet Bank El Qarya St., Off High Rd., Kafr el zayat, El gharbeya, KAFR EL ZAYAT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>الإلكترونيات</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -530,35 +530,35 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/599762</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/626132</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Target For Import And Export</t>
+          <t>OCEAN Mechanical Engineering</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>01110444615</t>
+          <t>01102631022</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>01110444615</t>
+          <t>01102631022</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>, 1St Industrial Zone, El katameya, Cairo, EL KATAMEYA</t>
+          <t>NASR CITY</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+          <t>الميكانيكا</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -568,35 +568,35 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/685213</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/685748</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Power System For Computer</t>
+          <t>Piece Of Art</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>01289601448</t>
+          <t>01015855587</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>01289601448</t>
+          <t>01015855587</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Mostafa El Araby St., El Koum El Akhdar, Faisal, Giza, FAISAL</t>
+          <t>Villa 116, , El Yasmeen 6 District, 1st Compound, New cairo, Cairo, NEW CAIRO</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -606,35 +606,35 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/424157</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/455619</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>El Hamd Service Center For Electronics &amp; Maintenance</t>
+          <t>Badawy Sons</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01224834563</t>
+          <t>01005152013</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>01224834563</t>
+          <t>01005152013</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Rd. 1, Ghebrial, Alexandria, GHEBRIAL</t>
+          <t>15 Mostafa Nassar St., Ain shams el sharkeya, Cairo, AIN SHAMS EL SHARKEYA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>الإلكترونيات</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -644,30 +644,30 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/392217</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/479514</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ebay</t>
+          <t>Green Fox For Computer</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>01007110210</t>
+          <t>01100087762</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>01007110210</t>
+          <t>01100087762</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>23 Ramsis St., El Korba, Heliopolis, Cairo, HELIOPOLIS</t>
+          <t>25 Misr Helwan Agricultural Rd., Maadi, Cairo, MAADI</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -682,35 +682,31 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/420237</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/621822</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>El Masa</t>
+          <t>Ideal House</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>01004994626</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>01004994626</t>
-        </is>
-      </c>
+          <t>0223521633</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Selim St., Koum Bakkar, Faisal, Giza, FAISAL</t>
+          <t>2 Ibrahim Nawar St., Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -720,35 +716,31 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/380508</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/468356</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>3M For Computer</t>
+          <t>Electro Mechanical Group - EMG</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>01140336393</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>01140336393</t>
-        </is>
-      </c>
+          <t>035482875</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>31 Gamal Abdel Nasser St. Farid Zaky Division, Hadayek helwan, Cairo, HADAYEK HELWAN</t>
+          <t>93 Mohamed Galal Hammad St., Miami, Alexandria, MIAMI</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الميكانيكا</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -758,35 +750,35 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/445117</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/452249</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ebtakarna Lak</t>
+          <t>Computer Shack</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>01000679000</t>
+          <t>01119536461</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>01000679000</t>
+          <t>01119536461</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>11 Palestine St., Off El Laselky St., Palestine Sq., New Maadi, Maadi, Cairo, MAADI</t>
+          <t>48 El Horreya St., Maadi, Cairo, MAADI</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -796,35 +788,35 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/616496</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/681219</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Saloni</t>
+          <t>Laptop Corner</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>01000255880</t>
+          <t>01033577195</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>01000255880</t>
+          <t>01033577195</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>, Customer Service, Heliopolis, Cairo, HELIOPOLIS</t>
+          <t>60 El Khalifa El Maamoun St., Mansheyet El Bakry, Heliopolis, Cairo, HELIOPOLIS</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -834,30 +826,26 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/425328</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/680479</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Alam El Computer Center</t>
+          <t>Winner Brands</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>01001808539</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>01001808539</t>
-        </is>
-      </c>
+          <t>035223316</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>9 Mahmoud Aref St, Off El Shishiny St., Faisal, Giza, FAISAL</t>
+          <t>36 Kafr Abdou St., Roushdy, Alexandria, ROUSHDY</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -872,35 +860,27 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/672789</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/395796</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Time Computer</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>01288111293</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>01288111293</t>
-        </is>
-      </c>
+          <t>Fawry Plus</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Eid Khairullah St., Agami, Alexandria, AGAMI</t>
+          <t>7 El Merryland Bldgs. Gesr El Suez St., Gesr el suez, Cairo, GESR EL SUEZ</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الإلكترونيات</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -910,30 +890,22 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/708464</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/633519</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Shaqawa</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>01004000146</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>01004000146</t>
-        </is>
-      </c>
+          <t>Electrotech For Computer</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>34 Awlad Ouf St., El Talbeya, El haram, Giza, EL HARAM</t>
+          <t>70 Ahmed Essmat St., Ain shams, Cairo, AIN SHAMS</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -948,30 +920,30 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/323509</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/482006</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sama For Computer</t>
+          <t>Mekka For Computer Services</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>01006965973</t>
+          <t>01004848500</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>01006965973</t>
+          <t>01004848500</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>28 El Gadid St., Kerdasa, Giza, Kerdasa</t>
+          <t>5 Saad Zaghloul St., Banha, Kaliobeya, BANHA</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -986,35 +958,35 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/558230</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/524159</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>El Tawhid For Computer</t>
+          <t>Misr Italia For Import And Export</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>01112853956</t>
+          <t>01012516852</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>01112853956</t>
+          <t>01012516852</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>70 Ain Shams St., Ain shams el sharkeya, Cairo, AIN SHAMS EL SHARKEYA</t>
+          <t>13 Joseph Tito St., El nozha el gadida, Cairo, EL NOZHA EL GADIDA</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1024,35 +996,27 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/377324</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/709254</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Smart Idea</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>01285266341</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>01285266341</t>
-        </is>
-      </c>
+          <t>WM Electronic</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>7 Amin El Leithy St., Amer City, Boulak el dakrour, Giza, BOULAK EL DAKROUR</t>
+          <t>2 El Hussein St., Off Ibn El Khattab St., Misr station, Alexandria, MISR STATION</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الإلكترونيات</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1062,27 +1026,35 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/447240</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/616777</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Mazloum Home</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
+          <t>Redline For Computer</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>01008290696</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>01008290696</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1 Mohamed Taimour St., Saint Fatima, Heliopolis, Cairo, HELIOPOLIS</t>
+          <t>18 El Bostan St., Bab el louk, Cairo, BAB EL LOUK</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1092,35 +1064,35 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/443149</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/556142</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Nour Steel For Restaurant And Hotel Equipment Supplies</t>
+          <t>Ebad El Rahman For Furniture</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>01222252311</t>
+          <t>01200357765</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>01222252311</t>
+          <t>01200357765</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Green Towers - Tower 6, Semouha, Alexandria, SEMOUHA</t>
+          <t>1 Khaled Ibn El Walid St., Hadayek El Maadi, Maadi, Cairo, MAADI</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1130,35 +1102,35 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/688235</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/504958</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>El Madina Furniture</t>
+          <t>Pro Solutions</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>01003933036</t>
+          <t>01096027500</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>01003933036</t>
+          <t>01096027500</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>38 Abbas Anany St., El badrashin, Giza, EL BADRASHIN</t>
+          <t>30 Gamal El Salakawy St.  Off Ahmed Maher St., Floor 1, El mansoura, El dakahleya, EL MANSOURA</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1168,30 +1140,26 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/606380</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/573426</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>El Walid For Computer</t>
+          <t>Escom</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>01099331470</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>01099331470</t>
-        </is>
-      </c>
+          <t>0482323969</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>7 Madraset El Motafaweqin St., Ain shams, Cairo, AIN SHAMS</t>
+          <t>Anwar El Sadat St. - El Galaa El Bahary St. Previously, Shebein el kawm, El monofeya, SHEBEIN EL KAWM</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1206,35 +1174,35 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/304663</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/322589</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>El Boraie For Coffee Shop Supplies</t>
+          <t>Adel Yehia Asal</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>01004358301</t>
+          <t>01228841541</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>01004358301</t>
+          <t>01228841541</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>8 Abou El Magd Abou Rehab St., Hadayek El Maadi, Maadi, Cairo, MAADI</t>
+          <t>38 El Karnak St., Faisal, Giza, FAISAL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1244,35 +1212,35 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/684571</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/340212</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RKB Plast</t>
+          <t>Square E For Electrical Industries</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>01224499742</t>
+          <t>01014591748</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>01224499742</t>
+          <t>01014591748</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>, Plastic Industrey Complex - Unit 17- 80, Mirghem, Alexandria, MIRGHEM</t>
+          <t>Factory No. 61, Industrial Zone C6, 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+          <t>الكهرباء والكابلات والأسلاك</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1282,35 +1250,35 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/690445</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/687960</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Abdou For Electronics Maintenance</t>
+          <t>Open Soft</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>01098912380</t>
+          <t>01099778997</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>01098912380</t>
+          <t>01099778997</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>29 Rd. 10, Zahraa Ain Shams, Ain shams el sharkeya, Cairo, AIN SHAMS EL SHARKEYA</t>
+          <t>El Mahgoub St., 3rd Neighbourhood, 1St District, New damietta, Damietta, NEW DAMIETTA</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>الإلكترونيات</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1320,35 +1288,27 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/653239</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/531486</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Al Mohtaseb Software</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>01024226678</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>01024226678</t>
-        </is>
-      </c>
+          <t>Upper Egypt Electricity Distribution Co.</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1 El Sheikh Mohamed El Nady St., Off Makram Ebaid St., 6th Zone, Nasr city, Cairo, NASR CITY</t>
+          <t>Misr Aswan Rd., El Odaisat, Luxor, Luxor, Luxor</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الكهرباء والكابلات والأسلاك</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1358,35 +1318,35 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/423840</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/672315</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Matrix For Computer Services</t>
+          <t>Nour El Sabah Showroom</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>01225661048</t>
+          <t>01003243970</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>01225661048</t>
+          <t>01003243970</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2 Othman Ibn Affan St., Kebaa city, Cairo, KEBAA CITY</t>
+          <t>98 Fayoum St., Dar el salam, Cairo, DAR EL SALAM</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1396,35 +1356,35 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/481671</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/331618</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>El Hagry For Computer</t>
+          <t>Qased Karim For Furniture</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>01126534898</t>
+          <t>01158667045</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>01126534898</t>
+          <t>01158667045</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>34 Dayer El Nahya St., Geziret Mohamed Village, El warak, Giza, EL WARAK</t>
+          <t>48 Mohamed Roshdy St., Ard El Haddad, Imbaba, Giza, IMBABA</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1434,26 +1394,30 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/599727</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/570857</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>High New Cairo Institute For Administrative Sciences &amp; Computer</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0222461112</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
+          <t>01273333282</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>01273333282</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>7th Neighbourhood, 1st Compound, New cairo, Cairo, NEW CAIRO</t>
+          <t>6 Abdel Qader El Rafaey St., Shoubra, Cairo, SHOUBRA</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1468,30 +1432,30 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/425132</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/432759</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>El Mokhtar Furniture</t>
+          <t>No Comment Furniture</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>01125923251</t>
+          <t>01210194499</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>01125923251</t>
+          <t>01210194499</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>125 El Gesr El Barrany St.  El Matbaa Sq., Dar el salam, Cairo, DAR EL SALAM</t>
+          <t>24 El Taqa St., 6th District, Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1506,30 +1470,22 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/507234</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/676360</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>VIP For Computer Services</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>01013799204</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>01013799204</t>
-        </is>
-      </c>
+          <t>Computer Shop</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>34 Abbas El Akkad St., Geziret el dahab, Giza, GEZIRET EL DAHAB</t>
+          <t>37 El Gomhoureya St., El mansoura, El dakahleya, EL MANSOURA</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1544,35 +1500,27 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/502498</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/545914</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>AM</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>01005055230</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>01005055230</t>
-        </is>
-      </c>
+          <t>Damson Furniture</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>41 Nasr Nassar St., Ard El Haddad, Imbaba, Giza, IMBABA</t>
+          <t>15 Mekka Towers Saad Zaghloul St., El Zohour District, Benisuef, Benisuef, Benisuef</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1582,35 +1530,35 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/353857</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/710010</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Stivan Furniture</t>
+          <t>El Barbary For Cars Electricity</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>01010183939</t>
+          <t>01117707950</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>01010183939</t>
+          <t>01117707950</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>, Service Spine, 11th District, 6th of october, Giza, 6th OF OCTOBER</t>
+          <t>6 El Tahrir St., El Shorbagy, Boulak el dakrour, Giza, BOULAK EL DAKROUR</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>الكهرباء والكابلات والأسلاك</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1620,22 +1568,30 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/668164</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/591577</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>E-Planet For Educational Services</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
+          <t>Caboo Play Station</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>01020104050</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>01020104050</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Sabry El Bekbashy St., Downtown, El fayoum, DOWNTOWN</t>
+          <t>31 Beacho American City Bldgs. El Haramain St., Phase 1, Zahraa El Maadi, Maadi, Cairo, MAADI</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1650,31 +1606,35 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/692021</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/640813</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Be Smart Solution</t>
+          <t>Online Furniture</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>035492386</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
+          <t>01121965179</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>01121965179</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2 El Mahdy St., Miami, Alexandria, MIAMI</t>
+          <t>Hassan Radwan St., Intersection Of Mostafa Fahmy St., Tanta, El gharbeya, TANTA</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1684,35 +1644,35 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/617353</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/639472</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Shahd &amp; Fady</t>
+          <t>Abou Yazan El Soury For Cars Electricity</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>01004009114</t>
+          <t>01154795368</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>01004009114</t>
+          <t>01154795368</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>El Shaheed Anwar St., El baragil, Giza, EL BARAGIL</t>
+          <t>El Kafrawy Spine, 2nd District, 6th of october, Giza, 6th OF OCTOBER</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الكهرباء والكابلات والأسلاك</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1722,31 +1682,27 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/348852</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/619415</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Global IT</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>0233807934</t>
-        </is>
-      </c>
+          <t>Upper Egypt Electricity Distribution Co.</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>76 Ahmed El Zayyat St., Dokki, Giza, DOKKI</t>
+          <t>, El Zaineya, LUXOR, Luxor, Luxor, Luxor</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الكهرباء والكابلات والأسلاك</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1756,30 +1712,26 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/671362</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/350737</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Collection For Furniture</t>
+          <t>Zebdaa For Goods &amp; Furniture Transport</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>01100315004</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>01100315004</t>
-        </is>
-      </c>
+          <t>0226820768</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>El Horreya St., Ezbet Khairallah, Dar el salam, Cairo, DAR EL SALAM</t>
+          <t>633 Port Said St., El Zaher Sq, First Of Kobry Ghamra, El zaher, Cairo, EL ZAHER</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1794,30 +1746,30 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/649260</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/440867</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Compu Lap Technology</t>
+          <t>Sama</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>01007905808</t>
+          <t>01116693396</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>01007905808</t>
+          <t>01116693396</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>136 El Hegaz St., Heliopolis, Cairo, HELIOPOLIS</t>
+          <t>30 El Masaken St., Faisal, Giza, FAISAL</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1832,26 +1784,30 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/426103</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/398156</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Soft Computer Services</t>
+          <t>Aqwad Software</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0653446555</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr"/>
+          <t>01277232772</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>01277232772</t>
+        </is>
+      </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>El Central El Seyahy St.  Off Sheraton Rd., Sekala, Hurghada, SEKALA</t>
+          <t>10 Fawzy Fahmy Gendy St.  Off Safeya Zagloul St., Raml station, Alexandria, RAML STATION</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1866,35 +1822,31 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/393763</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/485070</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>El Sharqawy Mall</t>
+          <t>Sharaf For Integrated Services</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>01221484651</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>01221484651</t>
-        </is>
-      </c>
+          <t>035732646</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>El Galaa St., Quwasnah, El monofeya, QUWASNAH</t>
+          <t>48 Khalil Ibrahim St., El Hoda Towers, Tower 4B, Ganaklis, Alexandria, GANAKLIS</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>أدوات النظافة</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1904,26 +1856,30 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/314343</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/575425</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Wizard For Computer Maintenance</t>
+          <t>Speed For Computer</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>035936026</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr"/>
+          <t>01155770771</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>01155770771</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>26 Adonis St., El ibrahimeya, Alexandria, EL IBRAHIMEYA</t>
+          <t>62 Salama Afify St., El zawia el hamra, Cairo, EL ZAWIA EL HAMRA</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -1938,35 +1894,27 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/473371</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/567492</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>El Hamd For Office Furniture</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>01095921098</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>01095921098</t>
-        </is>
-      </c>
+          <t>Fawry Plus</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Kobry El Adweya, El salam city, Cairo, EL SALAM CITY</t>
+          <t>1 Gamal Abdel Nasser St., Nasser, Benisuef, Nasser</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>الإلكترونيات</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1976,31 +1924,35 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/475708</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/698173</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Sobol Engineering Design Solutions</t>
+          <t>Defertec For Computer</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0221913371</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr"/>
+          <t>01066644197</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>01066644197</t>
+        </is>
+      </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>18 El Wehda El Arabeya St., Floor 2, Gesr el suez, Cairo, GESR EL SUEZ</t>
+          <t>126 Mostafa El Nahhas St., Floor 1, Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>الميكانيكا</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2010,35 +1962,31 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/539813</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/596769</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>El Adawy For Furniture</t>
+          <t>Global Wires</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>01112643615</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>01112643615</t>
-        </is>
-      </c>
+          <t>0224994045</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>abdel samea el haddad st., El Omraneya El Gharbeya, El haram, Giza, EL HARAM</t>
+          <t>31 Ain Shams St., Ain shams, Cairo, AIN SHAMS</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>الكهرباء والكابلات والأسلاك</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2048,35 +1996,27 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/314783</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/477097</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Concept For Furniture</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>01149360436</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>01149360436</t>
-        </is>
-      </c>
+          <t>Delta For Integrated Industries</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Plot 56, 1st District Services Zone, 5th Compound, New cairo, Cairo, NEW CAIRO</t>
+          <t>Plot 108, Industrial Zone B4, 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>أدوات النظافة</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2086,35 +2026,35 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/665389</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/456287</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Samer Shekhani For Restaurants Equipment</t>
+          <t>Umm El Qora Showroom</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>01112176687</t>
+          <t>01002307952</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>01112176687</t>
+          <t>01002307952</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>, El Hosary Sq., Central Spine, Alaa El Din Towers, Tower A, 7th District, 6th of october, Giza, 6th OF OCTOBER</t>
+          <t>El Omoumy St., Qalyub, Kaliobeya, QALYUB</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2124,30 +2064,30 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/644892</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/362854</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>El Khalil</t>
+          <t>El Shafaey</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>01004552797</t>
+          <t>01222218510</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>01004552797</t>
+          <t>01222218510</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Port Said St., As-santah, El gharbeya, AS-SANTAH</t>
+          <t>Abou Regaila St., Belqas, El dakahleya, BELQAS</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2162,35 +2102,35 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/349907</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/357664</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Technowow</t>
+          <t>Emago For Cleaning Services, General Supplies And Labor Supply</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>01013388535</t>
+          <t>01226629007</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>01013388535</t>
+          <t>01226629007</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>, Hadaeq October, Small Industries Compound, Bldg. 4, 6th of october, Giza, 6th OF OCTOBER</t>
+          <t>4 El Galaa St., Abdel Moneim Ryad Sq., Office 209, Downtown, Cairo, DOWNTOWN</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>أدوات النظافة</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2200,31 +2140,35 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/575148</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/709635</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Rayan Net Fom Computer</t>
+          <t>El Nouby</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>0238321196</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr"/>
+          <t>01062842716</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>01062842716</t>
+        </is>
+      </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>., 11th District, 6th of october, Giza, 6th OF OCTOBER</t>
+          <t>8 aioub st., Faggala, Cairo, FAGGALA</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2234,27 +2178,35 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/438046</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/325873</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Aman</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
+          <t>System Technology</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>01061833334</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>01061833334</t>
+        </is>
+      </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Gamal Abdel Nasser St., Nasser, Benisuef, Nasser</t>
+          <t>6 Moassaset El Zakah St., El marg, Cairo, EL MARG</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>الإلكترونيات</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2264,30 +2216,26 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/698560</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/481032</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Eyelets For Software</t>
+          <t>Jill Technology</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>01009996430</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>01009996430</t>
-        </is>
-      </c>
+          <t>0228713110</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>97 Khofo St.  Off Haram St., El haram, Giza, EL HARAM</t>
+          <t>28 Abdel Maaboud Yehia St., Off  El Kholafaa El Rashedin St., El marg, Cairo, EL MARG</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2302,7 +2250,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/540602</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/624717</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve error reporting and allow GET requests for scraper control
Update frontend to display specific error messages and switch scraper start/stop endpoints to support GET requests, alongside existing POST support.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 2a1fad78-d05e-42f0-ad61-6fa4ea0cba54
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 9a589ef7-04dc-4de3-838e-cb874d3efbbc
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/0ea4e3a5-1e4e-40d5-826b-5b1dabac3eb2/2a1fad78-d05e-42f0-ad61-6fa4ea0cba54/dSW4emr
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backup_temp.xlsx
+++ b/backup_temp.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,28 +461,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Hamis Fine Art</t>
+          <t>El Badr For Computer</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>01090013024</t>
+          <t>01005570863</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>01090013024</t>
+          <t>01005570863</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>12 Abou Bakr El Seddik St., El Mariouteya, Faisal, Giza, FAISAL</t>
+          <t>36 El Gadid St., Seriaqous, El khanka, Kaliobeya, EL KHANKA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -492,35 +492,35 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/454972</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/593052</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MG For Engineering &amp; Electronic Industries</t>
+          <t>Lamset Gamal Showroom</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>01225331212</t>
+          <t>01006726283</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>01225331212</t>
+          <t>01006726283</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1 Shonet Bank El Qarya St., Off High Rd., Kafr el zayat, El gharbeya, KAFR EL ZAYAT</t>
+          <t>267 Ahmed Zaky St., Hadayek El Maadi, Maadi, Cairo, MAADI</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>الإلكترونيات</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -530,35 +530,35 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/626132</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/418029</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>OCEAN Mechanical Engineering</t>
+          <t>Picks Office Furniture</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>01102631022</t>
+          <t>01091111812</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>01102631022</t>
+          <t>01091111812</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>NASR CITY</t>
+          <t>52 Emtedad Ramsis 2 El Nasr Rd., Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>الميكانيكا</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -568,35 +568,31 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/685748</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/677728</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Piece Of Art</t>
+          <t>El Naqaa For Computer</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>01015855587</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>01015855587</t>
-        </is>
-      </c>
+          <t>0238246759</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Villa 116, , El Yasmeen 6 District, 1st Compound, New cairo, Cairo, NEW CAIRO</t>
+          <t>Souad Kafafy St., El Motamayez District, 6th of october, Giza, 6th OF OCTOBER</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -606,30 +602,30 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/455619</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/440534</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Badawy Sons</t>
+          <t>Ahmed Abdel Daem For Furniture</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01005152013</t>
+          <t>01124423364</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>01005152013</t>
+          <t>01124423364</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15 Mostafa Nassar St., Ain shams el sharkeya, Cairo, AIN SHAMS EL SHARKEYA</t>
+          <t>30 El Mansheya St., Ezbet El Walda, Helwan, Cairo, HELWAN</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -644,35 +640,35 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/479514</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/483106</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Green Fox For Computer</t>
+          <t>El Mostafa Design</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>01100087762</t>
+          <t>01068882050</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>01100087762</t>
+          <t>01068882050</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>25 Misr Helwan Agricultural Rd., Maadi, Cairo, MAADI</t>
+          <t>El Mithaq St., Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -682,31 +678,35 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/621822</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/443026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ideal House</t>
+          <t>Power System For Computer</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0223521633</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>01289601448</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>01289601448</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2 Ibrahim Nawar St., Nasr city, Cairo, NASR CITY</t>
+          <t>Mostafa El Araby St., El Koum El Akhdar, Faisal, Giza, FAISAL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -716,31 +716,31 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/468356</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/424157</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Electro Mechanical Group - EMG</t>
+          <t>Star Link</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>035482875</t>
+          <t>0227043972</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>93 Mohamed Galal Hammad St., Miami, Alexandria, MIAMI</t>
+          <t>6 /13 El Gazaer St. 7th Sector, New Maadi, Maadi, Cairo, MAADI</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>الميكانيكا</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -750,35 +750,27 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/452249</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/373379</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Computer Shack</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>01119536461</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>01119536461</t>
-        </is>
-      </c>
+          <t>Fawry Plus</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>48 El Horreya St., Maadi, Cairo, MAADI</t>
+          <t>30 El Taawoneya Bldgs. El Lewaa Abdel Aziz Aly St. - El Mohafza St. Previously, El zagazig, El sharkeya, EL ZAGAZIG</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الإلكترونيات</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -788,35 +780,35 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/681219</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/633658</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Laptop Corner</t>
+          <t>Smart Vision</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>01033577195</t>
+          <t>01111226783</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>01033577195</t>
+          <t>01111226783</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>60 El Khalifa El Maamoun St., Mansheyet El Bakry, Heliopolis, Cairo, HELIOPOLIS</t>
+          <t>82 Mostafa El Nahhas St., Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -826,31 +818,35 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/680479</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/315098</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Winner Brands</t>
+          <t>Desouqy El Warraqy Furniture</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>035223316</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>01004550772</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>01004550772</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>36 Kafr Abdou St., Roushdy, Alexandria, ROUSHDY</t>
+          <t>26 Sidi Khamis St., Shebein el kawm, El monofeya, SHEBEIN EL KAWM</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -860,27 +856,35 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/395796</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/538086</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Fawry Plus</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
+          <t>El Ahleya</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>01005672822</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>01005672822</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>7 El Merryland Bldgs. Gesr El Suez St., Gesr el suez, Cairo, GESR EL SUEZ</t>
+          <t>El Morour Rd., Berket el sabaa, El monofeya, BERKET EL SABAA</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>الإلكترونيات</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -890,27 +894,35 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/633519</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/319610</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Electrotech For Computer</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
+          <t>Power For Engineering And Trade</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>01003194406</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>01003194406</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>70 Ahmed Essmat St., Ain shams, Cairo, AIN SHAMS</t>
+          <t>18 Ahmed Zakareya St., El Manar Mall, Downtown, Cairo, DOWNTOWN</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الكهرباء والكابلات والأسلاك</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -920,35 +932,31 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/482006</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/567933</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Mekka For Computer Services</t>
+          <t>El Amana For Electricity</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>01004848500</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>01004848500</t>
-        </is>
-      </c>
+          <t>0223917648</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>5 Saad Zaghloul St., Banha, Kaliobeya, BANHA</t>
+          <t>23 El Baidaq St., Ataba, Cairo, ATABA</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الكهرباء والكابلات والأسلاك</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -958,35 +966,31 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/524159</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/313879</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Misr Italia For Import And Export</t>
+          <t>Power Promaint For Integrated Maintenance</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>01012516852</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>01012516852</t>
-        </is>
-      </c>
+          <t>034700977</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>13 Joseph Tito St., El nozha el gadida, Cairo, EL NOZHA EL GADIDA</t>
+          <t>Km 23, Alex. cairo desert rd., Alexandria, ALEX. CAIRO DESERT RD.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+          <t>الميكانيكا</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -996,27 +1000,35 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/709254</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/631732</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>WM Electronic</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
+          <t>Guevara</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>01115276306</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>01115276306</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2 El Hussein St., Off Ibn El Khattab St., Misr station, Alexandria, MISR STATION</t>
+          <t>el hoda st., Dar el salam, Cairo, DAR EL SALAM</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>الإلكترونيات</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1026,30 +1038,30 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/616777</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/334708</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Redline For Computer</t>
+          <t>Malek For Technology Services</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>01008290696</t>
+          <t>01110559969</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>01008290696</t>
+          <t>01110559969</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>18 El Bostan St., Bab el louk, Cairo, BAB EL LOUK</t>
+          <t>El Dobbat Bldgs. Mostashfa El Kouat El Moussalha St., El salam city, Cairo, EL SALAM CITY</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1064,30 +1076,30 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/556142</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/644851</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ebad El Rahman For Furniture</t>
+          <t>Islam For Furniture</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>01200357765</t>
+          <t>01280932761</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>01200357765</t>
+          <t>01280932761</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1 Khaled Ibn El Walid St., Hadayek El Maadi, Maadi, Cairo, MAADI</t>
+          <t>15 Antar Hamzawy St., Bashteel Village, Auseem, Giza, AUSEEM</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1102,35 +1114,35 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/504958</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/544740</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pro Solutions</t>
+          <t>Youssef For Electronics</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>01096027500</t>
+          <t>01207779858</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>01096027500</t>
+          <t>01207779858</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>30 Gamal El Salakawy St.  Off Ahmed Maher St., Floor 1, El mansoura, El dakahleya, EL MANSOURA</t>
+          <t>21 El Teraa El Bahareya St., Umm Bayoumi, Shoubra el khaymah, Kaliobeya, SHOUBRA EL KHAYMAH</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الإلكترونيات</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1140,26 +1152,30 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/573426</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/473336</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Escom</t>
+          <t>Crazy Boy For Computer</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0482323969</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
+          <t>01144137167</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>01144137167</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Anwar El Sadat St. - El Galaa El Bahary St. Previously, Shebein el kawm, El monofeya, SHEBEIN EL KAWM</t>
+          <t>10 Masged El Tawhid St., Warraq El Arab, El warak, Giza, EL WARAK</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1174,35 +1190,35 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/322589</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/596683</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Adel Yehia Asal</t>
+          <t>El Mottahedoun</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>01228841541</t>
+          <t>01000264056</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>01228841541</t>
+          <t>01000264056</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>38 El Karnak St., Faisal, Giza, FAISAL</t>
+          <t>49 Noubar St., Bab el louk, Cairo, BAB EL LOUK</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1212,35 +1228,27 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/340212</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/306680</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Square E For Electrical Industries</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>01014591748</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>01014591748</t>
-        </is>
-      </c>
+          <t>IMAGE Home Department Store</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Factory No. 61, Industrial Zone C6, 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
+          <t>, Customer Service, Heliopolis, Cairo, HELIOPOLIS</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>الكهرباء والكابلات والأسلاك</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1250,35 +1258,35 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/687960</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/509252</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Open Soft</t>
+          <t>Queen Furniture &amp; Decoration</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>01099778997</t>
+          <t>01113823818</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>01099778997</t>
+          <t>01113823818</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>El Mahgoub St., 3rd Neighbourhood, 1St District, New damietta, Damietta, NEW DAMIETTA</t>
+          <t>Military Academy Wall Othman Ibn Affan St., Heliopolis, Cairo, HELIOPOLIS</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1288,14 +1296,14 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/531486</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/680378</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Upper Egypt Electricity Distribution Co.</t>
+          <t>Aman</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -1303,12 +1311,12 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Misr Aswan Rd., El Odaisat, Luxor, Luxor, Luxor</t>
+          <t>25 El Tahrir St., Bab el louk, Cairo, BAB EL LOUK</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>الكهرباء والكابلات والأسلاك</t>
+          <t>الإلكترونيات</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1318,35 +1326,31 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/672315</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/578716</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Nour El Sabah Showroom</t>
+          <t>El Masreya For Electronics Devices Maintenance</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>01003243970</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>01003243970</t>
-        </is>
-      </c>
+          <t>0223866783</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>98 Fayoum St., Dar el salam, Cairo, DAR EL SALAM</t>
+          <t>13 Omar Zaafan St., 1st Zone, Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>الإلكترونيات</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1356,30 +1360,30 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/331618</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/313501</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Qased Karim For Furniture</t>
+          <t>Stark Office Furniture</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>01158667045</t>
+          <t>01201155022</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>01158667045</t>
+          <t>01201155022</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>48 Mohamed Roshdy St., Ard El Haddad, Imbaba, Giza, IMBABA</t>
+          <t>1 /3 El Laselky St., New Maadi, Maadi, Cairo, MAADI</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1394,35 +1398,35 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/570857</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/463548</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>Meki Electromechanical &amp; Construction - Meecon</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>01273333282</t>
+          <t>01066230148</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>01273333282</t>
+          <t>01066230148</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>6 Abdel Qader El Rafaey St., Shoubra, Cairo, SHOUBRA</t>
+          <t>27 El Kholafaa El Rashedeen St.,, Tanta, El gharbeya, TANTA</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الميكانيكا</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1432,35 +1436,31 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/432759</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/674330</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>No Comment Furniture</t>
+          <t>Nascom - Egyptian Co. For Supplies &amp; Contracting</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>01210194499</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>01210194499</t>
-        </is>
-      </c>
+          <t>0233363670</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>24 El Taqa St., 6th District, Nasr city, Cairo, NASR CITY</t>
+          <t>Plot 10, Northern Extensions, Polaris International Zone, 6th of october, Giza, 6th OF OCTOBER</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>الميكانيكا</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1470,14 +1470,14 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/676360</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/694042</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Computer Shop</t>
+          <t>Forbed</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1485,12 +1485,12 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>37 El Gomhoureya St., El mansoura, El dakahleya, EL MANSOURA</t>
+          <t>, Ard El Mahlag, As sinbillawain, El dakahleya, AS SINBILLAWAIN</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1500,14 +1500,14 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/545914</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/713251</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Damson Furniture</t>
+          <t>Aman</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1515,12 +1515,12 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>15 Mekka Towers Saad Zaghloul St., El Zohour District, Benisuef, Benisuef, Benisuef</t>
+          <t>2 El Nasser Salah El Din St., Off El Tahrir St., Kom hamada, El beheira, KOM HAMADA</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>الإلكترونيات</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1530,35 +1530,31 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/710010</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/632401</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>El Barbary For Cars Electricity</t>
+          <t>Arment Secondary For Mechanical Works For Boys</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>01117707950</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>01117707950</t>
-        </is>
-      </c>
+          <t>0952481045</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>6 El Tahrir St., El Shorbagy, Boulak el dakrour, Giza, BOULAK EL DAKROUR</t>
+          <t>Hager Abou Qolaiey Village, Arment, Luxor, Arment</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>الكهرباء والكابلات والأسلاك</t>
+          <t>الميكانيكا</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1568,30 +1564,30 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/591577</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/365767</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Caboo Play Station</t>
+          <t>AMS Mikrotik</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>01020104050</t>
+          <t>01090201477</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>01020104050</t>
+          <t>01090201477</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>31 Beacho American City Bldgs. El Haramain St., Phase 1, Zahraa El Maadi, Maadi, Cairo, MAADI</t>
+          <t>, Freelance Business, Moharram bey, Alexandria, MOHARRAM BEY</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1606,35 +1602,35 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/640813</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/545686</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Online Furniture</t>
+          <t>Abou Elainen Mattar Sons For Gas Ovens</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>01121965179</t>
+          <t>01111646070</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>01121965179</t>
+          <t>01111646070</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Hassan Radwan St., Intersection Of Mostafa Fahmy St., Tanta, El gharbeya, TANTA</t>
+          <t>, Deyrb Negm Rd., Sentamay, Mit ghamr, El dakahleya, MIT GHAMR</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1644,35 +1640,35 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/639472</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/685642</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Abou Yazan El Soury For Cars Electricity</t>
+          <t>Kasr El Malek Showroom</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>01154795368</t>
+          <t>01225314223</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>01154795368</t>
+          <t>01225314223</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>El Kafrawy Spine, 2nd District, 6th of october, Giza, 6th OF OCTOBER</t>
+          <t>El Gharby St., Helwan, Cairo, HELWAN</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>الكهرباء والكابلات والأسلاك</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1682,27 +1678,31 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/619415</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/385944</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Upper Egypt Electricity Distribution Co.</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
+          <t>Procoor International</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0223084552</t>
+        </is>
+      </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>, El Zaineya, LUXOR, Luxor, Luxor, Luxor</t>
+          <t>Villa 18, Banafseg, New cairo, Cairo, NEW CAIRO</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>الكهرباء والكابلات والأسلاك</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1712,26 +1712,26 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/350737</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/606581</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Zebdaa For Goods &amp; Furniture Transport</t>
+          <t>Selection</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0226820768</t>
+          <t>0403400164</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>633 Port Said St., El Zaher Sq, First Of Kobry Ghamra, El zaher, Cairo, EL ZAHER</t>
+          <t>El Fateh St. Off Othman Ibn Affan St., Tanta, El gharbeya, TANTA</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1746,30 +1746,30 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/440867</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/437683</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Sama</t>
+          <t>International Technology</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>01116693396</t>
+          <t>01229213654</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>01116693396</t>
+          <t>01229213654</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>30 El Masaken St., Faisal, Giza, FAISAL</t>
+          <t>7 Ibrahim Zanaty St. Off Selim El Awal St., El zaytoun, Cairo, EL ZAYTOUN</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1784,30 +1784,26 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/398156</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/466651</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Aqwad Software</t>
+          <t>El Mobtakeron</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>01277232772</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>01277232772</t>
-        </is>
-      </c>
+          <t>0222876817</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>10 Fawzy Fahmy Gendy St.  Off Safeya Zagloul St., Raml station, Alexandria, RAML STATION</t>
+          <t>135 Mostafa El Nahhas St., Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1822,31 +1818,35 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/485070</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/453791</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Sharaf For Integrated Services</t>
+          <t>El Shorouq Furniture</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>035732646</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr"/>
+          <t>01005104922</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>01005104922</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>48 Khalil Ibrahim St., El Hoda Towers, Tower 4B, Ganaklis, Alexandria, GANAKLIS</t>
+          <t>20 Teraet El Sisy St., El Mariouteya, El haram, Giza, EL HARAM</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>أدوات النظافة</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1856,30 +1856,22 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/575425</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/508239</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Speed For Computer</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>01155770771</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>01155770771</t>
-        </is>
-      </c>
+          <t>2B Egypt</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>62 Salama Afify St., El zawia el hamra, Cairo, EL ZAWIA EL HAMRA</t>
+          <t>200 El Nozha St., Hegaz Square, Heliopolis, Cairo, HELIOPOLIS</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -1894,27 +1886,31 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/567492</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/692040</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Fawry Plus</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr"/>
+          <t>El Masry For General Supplies</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>0235705657</t>
+        </is>
+      </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1 Gamal Abdel Nasser St., Nasser, Benisuef, Nasser</t>
+          <t>38 Rabea El Gizy St., Giza Administrative Tower, Floor 4, Giza, Giza, GIZA</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>الإلكترونيات</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1924,35 +1920,27 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/698173</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/353330</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Defertec For Computer</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>01066644197</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>01066644197</t>
-        </is>
-      </c>
+          <t>Forbed</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>126 Mostafa El Nahhas St., Floor 1, Nasr city, Cairo, NASR CITY</t>
+          <t>El Gamea El Kabir St., El hamoul, Kafr el sheikh, EL HAMOUL</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1962,31 +1950,35 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/596769</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/713256</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Global Wires</t>
+          <t>Mazaya For Computer</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0224994045</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr"/>
+          <t>01100276377</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>01100276377</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>31 Ain Shams St., Ain shams, Cairo, AIN SHAMS</t>
+          <t>7 Sphinx Sq., Mohandeseen, Giza, MOHANDESEEN</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>الكهرباء والكابلات والأسلاك</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1996,27 +1988,35 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/477097</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/461619</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Delta For Integrated Industries</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
+          <t>Future Power</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>01281861008</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>01281861008</t>
+        </is>
+      </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Plot 108, Industrial Zone B4, 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
+          <t>26 Naguib El Rihany St., Downtown, Cairo, DOWNTOWN</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>أدوات النظافة</t>
+          <t>الكهرباء والكابلات والأسلاك</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2026,30 +2026,30 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/456287</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/708387</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Umm El Qora Showroom</t>
+          <t>Al-Ashry for Home, Office, and Chalet Furniture</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>01002307952</t>
+          <t>01000171870</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>01002307952</t>
+          <t>01000171870</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>El Omoumy St., Qalyub, Kaliobeya, QALYUB</t>
+          <t>Borg El Arab City Entrance - Main Road, New borg el arab, Alexandria, NEW BORG EL ARAB</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2064,30 +2064,22 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/362854</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/501499</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>El Shafaey</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>01222218510</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>01222218510</t>
-        </is>
-      </c>
+          <t>2B Egypt</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Abou Regaila St., Belqas, El dakahleya, BELQAS</t>
+          <t>Omar Ibn El Khattab St., Nasr city, Cairo, NASR CITY</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2102,35 +2094,31 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/357664</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/331276</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Emago For Cleaning Services, General Supplies And Labor Supply</t>
+          <t>El Saada</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>01226629007</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>01226629007</t>
-        </is>
-      </c>
+          <t>0242154633</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>4 El Galaa St., Abdel Moneim Ryad Sq., Office 209, Downtown, Cairo, DOWNTOWN</t>
+          <t>10th of ramadan st., Qalyub, Kaliobeya, QALYUB</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>أدوات النظافة</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2140,30 +2128,30 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/709635</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/303599</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>El Nouby</t>
+          <t>El Meniawy</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>01062842716</t>
+          <t>01285449292</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>01062842716</t>
+          <t>01285449292</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>8 aioub st., Faggala, Cairo, FAGGALA</t>
+          <t>14 Teraet El Gallad St., El zawia el hamra, Cairo, EL ZAWIA EL HAMRA</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2178,35 +2166,35 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/325873</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/411243</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>System Technology</t>
+          <t>El Asiouty Furniture</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>01061833334</t>
+          <t>01118206136</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>01061833334</t>
+          <t>01118206136</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>6 Moassaset El Zakah St., El marg, Cairo, EL MARG</t>
+          <t>El Hosary Sq., Central Spine, 7th District, 6th of october, Giza, 6th OF OCTOBER</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2216,41 +2204,1861 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/481032</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/599007</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Jill Technology</t>
+          <t>Abou Ahmed For Furniture Paints</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>0228713110</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr"/>
+          <t>01128389981</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>01128389981</t>
+        </is>
+      </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>28 Abdel Maaboud Yehia St., Off  El Kholafaa El Rashedin St., El marg, Cairo, EL MARG</t>
+          <t>1 El Mohandes Nouh Aly Hussein St., El bassateen, Cairo, EL BASSATEEN</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/684767</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Computec</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>01093166993</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>01093166993</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>33 /32 Hasab Allah El Kafrawy St.  3rd Neighbourhood, 2nd District, New damietta, Damietta, NEW DAMIETTA</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
           <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>YellowPages</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/624717</t>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/529024</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Rich Home</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>035912860</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>12 Omar Zaafan St., El ibrahimeya, Alexandria, EL IBRAHIMEYA</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/301899</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Taha For Furniture Paints</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>01066961055</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>01066961055</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>34 Mohamed Khalifa St., Hadayek El Maadi, Maadi, Cairo, MAADI</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/676811</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Furniture World</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>0233025296</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Abdel Wahed Hassan St., Agouza, Giza, AGOUZA</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/393509</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>El Omaraa</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>01003528566</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>01003528566</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Tanan Village, Qalyub, Kaliobeya, QALYUB</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/363429</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>El Shamel For Computer Services</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>01094936836</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>01094936836</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>7 Madraset El Motafaweqin St., Ain shams, Cairo, AIN SHAMS</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/626673</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Fawry Plus</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>, Central Spine, El Hosary Sq., Bldg. 40, 2nd District, 6th of october, Giza, 6th OF OCTOBER</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>الإلكترونيات</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/633250</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Project Egy</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>01096886288</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>01096886288</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>336 Faisal St., Faisal, Giza, FAISAL</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/678229</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Abou Gad For Furniture</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>01118565601</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>01118565601</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>25 El Guish St., El Ezba El Sharqeya, El hawamdeya, Giza, EL HAWAMDEYA</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/615033</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>El Masreya For Fire Fighting Systems</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>01280115249</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>01280115249</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>El Guish St. Off 23rd Of July St., Arish, North sinai, ARISH</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>الصحة والسلامة ومقاومة الحريق</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/526470</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>My Computer</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>0233756984</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>1 El Samah St., Off El Madrasa St., El moneeb, Giza, EL MONEEB</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/413005</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Omoula For Furniture</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>01153812908</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>01153812908</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>14 Naguib Mahfouz St., Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/683011</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>01062507185</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>01062507185</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Abdel Salam Aref St., El shohadaa, El monofeya, El Shohadaa</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/314150</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>EPC Solutions</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>0222699470</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>42 A Autostrad Rd., El Moltaqa El Araby District, Floor 1  Flat 102, Sheraton Bldgs., Heliopolis, Cairo, HELIOPOLIS</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>الصحة والسلامة ومقاومة الحريق</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/574408</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>01061686523</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>01061686523</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>el maleka st., Faisal, Giza, FAISAL</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/341381</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>East Asia</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Mostafa Kamel St., Semouha, Alexandria, SEMOUHA</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/678868</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Ice &amp; Fire For Computer</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>01228408763</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>01228408763</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>2 El Khosous El Omoumy St., El khosous, Kaliobeya, EL KHOSOUS</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/499521</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Barcelona For Computer</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>01221241553</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>01221241553</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>1 Abou Bakr El Seddik St.  Off Mahmoud Ammar St., Ezbet El Hagana, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/310043</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Egyptian Workshop</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>01005234875</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>01005234875</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>10 Sayed Abou Emaira St., El haram, Giza, EL HARAM</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>الصحة والسلامة ومقاومة الحريق</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/320607</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Top Technology</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>0224124823</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>petroleum Bldgs.,, 10th District, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/310329</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Travel Maker Trips</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>01286783479</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>01286783479</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>2 Mohamed Ahmed St., Flat 303, Floor 3, Off Ahmed Badawy St., Shoubra, Cairo, SHOUBRA</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/625925</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Blue Code</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>01555568631</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>01555568631</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>26 Gamaet El Dewal El Arabeya St., Mohandeseen, Giza, MOHANDESEEN</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/714281</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Al Fannia Co. For Hotels Supplies</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>0227861705</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>2 Naguib El Rihany St., Intersection Of Clot Bey St., Downtown, Cairo, DOWNTOWN</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/535480</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>El Qods</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>01011220043</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>01011220043</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>El Tahrir St., Kafr sakr, El sharkeya, KAFR SAKR</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/351912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Al Ethad Company For Industrial Security Equipment And Firefighting Systems</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>0453286015</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>El Mrour St., Off Cairo Alex Agricultural Rd., Damanhour, El beheira, Damanhour</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>الصحة والسلامة ومقاومة الحريق</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/696044</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>El Hamd For Electromechanical Supplies</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>01116960269</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>01116960269</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>, El Ordoneya, City Center, 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>الميكانيكا</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/619766</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>X Game Stores</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>01000138959</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>01000138959</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Km 52 Misr Ismaileya Desert Rd., 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/669320</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Bedaya For Computer</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>01010016188</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>01010016188</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>43 El Eshreen St., Saft El Laban, Boulak el dakrour, Giza, BOULAK EL DAKROUR</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/579237</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>3 Kharabish St., Belbeis, El sharkeya, BELBEIS</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>الإلكترونيات</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/632408</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Nour Computer Center</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>01004168876</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>01004168876</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>3 Hashem El Wafaey St., Faisal, Giza, FAISAL</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/397214</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>El Sonbaty Modern</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>01111063203</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>01111063203</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>., 5th District, 6th of october, Giza, 6th OF OCTOBER</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/359090</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Compu Nour</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>01116489768</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>01116489768</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>110 Ibrahim Abdel Razeq St., Ain shams, Cairo, AIN SHAMS</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/416836</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>El Etmany For Furniture</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>01064727175</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>01064727175</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>5 Awlad El Gamal St,, Off Abdel Hamid Mekky St., Hadayek El Maadi, Maadi, Cairo, MAADI</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/686066</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Living In Interiors</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>0227262021</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Plot 202, 2nd Sector, 5th Compound, New cairo, Cairo, NEW CAIRO</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/431680</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Teradata</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>0237764500</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>21 Giza St., Giza, Giza, GIZA</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/437942</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>El Sabereen For Computer Services</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>01006532006</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>01006532006</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Warshet El Balat St., Agami, Alexandria, AGAMI</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/396235</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Kasr El Sultan For Furniture</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>01007841117</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>01007841117</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>109 Teraet Abdel Aal 2 St., Saft El Laban, Boulak el dakrour, Giza, BOULAK EL DAKROUR</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/579266</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Kabbani Furniture</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr"/>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>30 Salah El Din El Aiouby St., Assyout, Assyout, Assyout</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/689648</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Abou Shahen</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>01224326828</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>01224326828</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>35 El Bokhary St., 7th District, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/314966</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr"/>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>107 Masged El Seddik St., El bitash, Alexandria, EL BITASH</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>الإلكترونيات</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/698086</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Abdel Malek For Furniture</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>01270009595</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>01270009595</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>18 Sudan St., Mohandeseen, Giza, MOHANDESEEN</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/464213</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Hamada For Computer</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>01112550207</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>01112550207</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>26 Gamal Abdel Nasser St., Kafr Berak El Khayyam, Boulak el dakrour, Giza, BOULAK EL DAKROUR</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/556736</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Viola For Furniture</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>01066223999</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>01066223999</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>26 El Thawra St., Almaza, Heliopolis, Cairo, HELIOPOLIS</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/683163</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>A &amp; M</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>01285252688</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>01285252688</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>15 Mamdouh Ramadan St.  Off El Safa W El Marwa, El Tawabeq, Faisal, Giza, FAISAL</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/470896</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Mohamed Workshop</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>01229909121</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>01229909121</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>El Zahaby St., Qalyub, Kaliobeya, QALYUB</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/363498</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>El Madina El Monawara For Computer Services</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>01069690025</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>01069690025</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>1 Refaat Abdel Fattah St., El Talbeya, El haram, Giza, EL HARAM</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/639383</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Vitrine Furniture</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>01120210077</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>01120210077</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>, Mohamed Naguib Spine, 5th Compound, New cairo, Cairo, NEW CAIRO</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/709995</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>El Mostafa For Furniture</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>01229196740</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>01229196740</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>8 Hussein Ibrahim St., El herafeyeen, Cairo, EL HERAFEYEEN</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/478212</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>El Swedy For Cables</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>01020510151</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>01020510151</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>, Sector 13, Bldg. 1, Zahraa El Maadi, Maadi, Cairo, MAADI</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/686961</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Fawry Plus</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr"/>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>42 Mossadak St., Dokki, Giza, DOKKI</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>الإلكترونيات</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/633482</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace long configuration URLs with compact bitmask encoding
Update API endpoints to use bitmask encoding for scraper configuration, replacing lengthy base64 encoded URLs to prevent proxy request length limitations.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 7e3d5077-08fc-4c45-89fc-edb63a29d7de
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 2f577417-eeb2-4363-ab32-405503effed8
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/e3daa699-cb02-4e21-8269-a67f6b6deaa8/7e3d5077-08fc-4c45-89fc-edb63a29d7de/FezNkVd
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backup_temp.xlsx
+++ b/backup_temp.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,29 +471,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>El Mona Center For Physiotherapy</t>
+          <t>Zahabeya</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>01006861578</t>
+          <t>01118383013</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>01006861578</t>
+          <t>01118383013</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>El Leithy St., Mit ghamr, El dakahleya, MIT GHAMR</t>
+          <t>Atlas St., Helwan, Cairo, HELWAN</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأغذية والمشروبات</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -508,36 +508,36 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/337522</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/335805</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tiba</t>
+          <t>Yopie Fries</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>01146670392</t>
+          <t>01203984004</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>01146670392</t>
+          <t>01203984004</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Lailat El Qadr Sq., 6th of october, Giza, 6th OF OCTOBER</t>
+          <t>Dokki St., Dokki, Giza, DOKKI</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>السيارات وقطع الغيار</t>
+          <t>الأغذية والمشروبات</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -552,32 +552,32 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/438960</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/691335</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Master Tech</t>
+          <t>Slash Group For Trade</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0242211431</t>
+          <t>0233930395</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Abdullah Ewais St., Shoubra el khaymah, Kaliobeya, SHOUBRA EL KHAYMAH</t>
+          <t>8 Hassan Hebaish St., Floor 4, Off Madkour St., Madkour, El haram, Giza, EL HARAM</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأغذية والمشروبات</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -592,41 +592,37 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/413951</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/359682</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ahmed Abou Delaa For Advertising</t>
+          <t>Genos</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>01226424538</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>01226424538</t>
-        </is>
-      </c>
+          <t>0235834502</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2 Omar Ibn El Khattab St., El khosous, Kaliobeya, EL KHOSOUS</t>
+          <t>259 Haram St., El haram, Giza, EL HARAM</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>الطباعة والنشر والإعلان</t>
+          <t>الأغذية والمشروبات</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>📱 واتساب فقط</t>
+          <t>☎ هاتف فقط</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -636,36 +632,36 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/494415</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/391457</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Lady Lingerie</t>
+          <t>Delta Pharma</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01200316609</t>
+          <t>01066630591</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>01200316609</t>
+          <t>01066630591</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Alex Matrouh Desert Rd., Agami, Alexandria, AGAMI</t>
+          <t>Km 81, Cairo Alex Desert Rd., El noubareya, El beheira, EL NOUBAREYA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>النسيج والملابس</t>
+          <t>الزراعة والري</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -680,33 +676,41 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/430527</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/487554</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Daddy's Burger</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
+          <t>El Maher Satellite</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>01115401100</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>01115401100</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>37 A El Tesaeen El Shamaly St., 5th Compound, New cairo, Cairo, NEW CAIRO</t>
+          <t>2 B El Khamseen St., Mansheyet Gebril Division, Zahraa El Maadi, Maadi, Cairo, MAADI</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>الأغذية والمشروبات</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>📱 واتساب فقط</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -716,32 +720,32 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/570088</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/461649</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>El Seoudi Establishment For Trading &amp; Contracting</t>
+          <t>United Marine Surveyors</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0224040186</t>
+          <t>034843385</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4 El Obour Bldgs. Salah Salem Rd., Floor 4, Heliopolis, Cairo, HELIOPOLIS</t>
+          <t>9 Abou El Nasr St.  Off Kasr Ras El Teen St., Floor 3, Bahary, Alexandria, BAHARY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>مواد البناء والمقاولات</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -756,36 +760,36 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/464916</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/429934</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>El Arkan For Medical Supplies</t>
+          <t>Durban For Clothes</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>01066610714</t>
+          <t>01008200599</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>01066610714</t>
+          <t>01008200599</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>31 El Batal Ahmed Abdel Aziz St., Mohandeseen, Giza, MOHANDESEEN</t>
+          <t>74 El Horreya St., Helmeyet el zaitoun, Cairo, HELMEYET EL ZAITOUN</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>المعدات الطبية والصيدلانية</t>
+          <t>النسيج والملابس</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -800,36 +804,36 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/663055</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/660227</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Software For Satellite</t>
+          <t>Mr Burger</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>01128588621</t>
+          <t>01277444092</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>01128588621</t>
+          <t>01277444092</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2 Masged Namera St., Hadayek El Maadi, Maadi, Cairo, MAADI</t>
+          <t>45 Aziz Antoine St., El seyouf shamaa, Alexandria, EL SEYOUF SHAMAA</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأغذية والمشروبات</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -844,14 +848,14 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/684566</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/637647</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Concrete</t>
+          <t>October For Development &amp; Real Estate Investment</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -859,13 +863,13 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Omar Ibn El Khattab St., Nasr city, Cairo, NASR CITY</t>
+          <t>, Customer Service, Dokki, Giza, DOKKI</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>النسيج والملابس</t>
+          <t>العقارات والمقاولات</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -880,30 +884,30 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/696403</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/545782</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Fruit Paradise</t>
+          <t>El Saidy Sons For Sanitary Ware</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>01550771626</t>
+          <t>01126959220</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>01550771626</t>
+          <t>01126959220</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>67 Safeya Zaghloul St., Raml station, Alexandria, RAML STATION</t>
+          <t>10 Tanta St., Off Mohamed Mostafa El Sherif St., Ezbet el nakhl, Cairo, EZBET EL NAKHL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -924,36 +928,36 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/582453</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/533021</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Techincal Workshop For Cars Repairing</t>
+          <t>Aman Labs For Medical Analysis &amp; Blood Research</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>01098319823</t>
+          <t>01006906486</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>01098319823</t>
+          <t>01006906486</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>12 Abou Serea El Ghobashy St., Zahraa Ain Shams, Ain shams, Cairo, AIN SHAMS</t>
+          <t>1 El Thawra St., Off Hassanein Desouqy St., Hadayek El Maadi, Maadi, Cairo, MAADI</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>السيارات وقطع الغيار</t>
+          <t>المعدات الطبية والصيدلانية</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -968,41 +972,33 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/650768</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/506672</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abou Eissa For Clothes</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>01285401816</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>01285401816</t>
-        </is>
-      </c>
+          <t>Manna Patisserie</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>6 Dayer El Nahya St., Saft El Laban, Boulak el dakrour, Giza, BOULAK EL DAKROUR</t>
+          <t>Syria St., Roushdy, Alexandria, ROUSHDY</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>النسيج والملابس</t>
+          <t>الأغذية والمشروبات</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>📱 واتساب فقط</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1012,36 +1008,36 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/579104</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/339797</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>El Tawhid</t>
+          <t>El Rahma Center For Satellite</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>01229555046</t>
+          <t>01100608187</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>01229555046</t>
+          <t>01100608187</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>el maasarawy st., El Omraneya El Sharkeya, El haram, Giza, EL HARAM</t>
+          <t>82 El Wehda El Arabia St., Gesr el suez, Cairo, GESR EL SUEZ</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>الأغذية والمشروبات</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1056,26 +1052,30 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/308530</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/653495</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ETA - Engineering Trade Association</t>
+          <t>Puzzle Advertising &amp; Marketing Solutions</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0227009155</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
+          <t>01226009955</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>01226009955</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>32 El Shorta Towers, Autostrad Rd., El Amal City, New Maadi, Maadi, Cairo, MAADI</t>
+          <t>46 El Nozha St., El Sheikh Zayed, 6th of october, Giza, 6th OF OCTOBER</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -1086,7 +1086,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>☎ هاتف فقط</t>
+          <t>📱 واتساب فقط</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1096,22 +1096,30 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/512472</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/538948</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Nos Dasta</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
+          <t>El Horany Fish</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>01211130303</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>01211130303</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Wezaret El Zeraah St., Dokki, Giza, DOKKI</t>
+          <t>Nady El Seid St., Dokki, Giza, DOKKI</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -1122,7 +1130,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>📱 واتساب فقط</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1132,41 +1140,37 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/694839</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/678784</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashraqt</t>
+          <t>El Mohandes</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>01282914050</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>01282914050</t>
-        </is>
-      </c>
+          <t>0224552001</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>El Emam El Shaarawy St., Mit ghamr, El dakahleya, MIT GHAMR</t>
+          <t>12 Dar El Salam St., Saray el koba, Cairo, SARAY EL KOBA</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>النسيج والملابس</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>📱 واتساب فقط</t>
+          <t>☎ هاتف فقط</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1176,30 +1180,22 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/339597</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/399855</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Dr. Ashraf Haidar Laboratory</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>01007501079</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>01007501079</t>
-        </is>
-      </c>
+          <t>Al Shams Labs</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>123 Kamal El Shazly St. - El Guish St. Previously, El bagour, El monofeya, EL BAGOUR</t>
+          <t>9 Said Zou El Foqqar St., El Pasha Sq., El manyal, Cairo, EL MANYAL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -1210,7 +1206,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>📱 واتساب فقط</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1220,36 +1216,36 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/559253</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/443364</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Baid El Maeda</t>
+          <t>Abou Hala Furniture Moving</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>01140333272</t>
+          <t>01001212408</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>01140333272</t>
+          <t>01001212408</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>El Sahran Bldgs., Block 6, Gesr El Manawat St., El hawamdeya, Giza, EL HAWAMDEYA</t>
+          <t>HELIOPOLIS</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>الأغذية والمشروبات</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1264,36 +1260,36 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/604627</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/685984</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>El Motaheda For Cars Maintenance</t>
+          <t>Cheesy Pan</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>01003894068</t>
+          <t>01033369777</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>01003894068</t>
+          <t>01033369777</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>3 El Awqaf Investment Towers, El Rashah St., Qalyub, Kaliobeya, QALYUB</t>
+          <t>El Khamseen St., Sector 13, Zahraa El Maadi, Maadi, Cairo, MAADI</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>السيارات وقطع الغيار</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1308,36 +1304,36 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/527365</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/609192</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Specialist Transport Services &amp; Logistics Business</t>
+          <t>Dr. Micheal George Boabgian Lab</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>01555557892</t>
+          <t>01222116631</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>01555557892</t>
+          <t>01222116631</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>4 O El Wozaraa Square, Plot 1166, Sheraton Bldgs., Heliopolis, Cairo, HELIOPOLIS</t>
+          <t>102 B El Merghany St., Heliopolis, Cairo, HELIOPOLIS</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>الشحن والنقل واللوجستيات</t>
+          <t>المعدات الطبية والصيدلانية</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1352,30 +1348,30 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/545983</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/425133</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Gawharet El Madina El Haditha For Gifts</t>
+          <t>Global For Accounting &amp; Auditing</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>01123221449</t>
+          <t>01287804623</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>01123221449</t>
+          <t>01287804623</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3 Ibrahim Madkour St., Abou el nomrous, Giza, Abou El Nomrous</t>
+          <t>, 75 Neighborhood, Green View Compound, 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -1396,36 +1392,36 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/602818</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/694269</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Golden Apple Group For Trade, Industry &amp; Construction</t>
+          <t>El Maghraby For Air Condition</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>01228980002</t>
+          <t>01287032705</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>01228980002</t>
+          <t>01287032705</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Block 23 - Plot 8, , 4th Industrial Zone, Borg el arab, Alexandria, BORG EL ARAB</t>
+          <t>el morour st., Berket el sabaa, El monofeya, BERKET EL SABAA</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>مواد البناء والمقاولات</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1440,36 +1436,36 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/598751</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/319881</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Misr Italia For Kitchens</t>
+          <t>Everest For Office Furniture</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>01005711424</t>
+          <t>01064150700</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>01005711424</t>
+          <t>01064150700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>49 A Abbas El Akkad St., 1st Zone, Nasr city, Cairo, NASR CITY</t>
+          <t>123 Faisal St., El Koum El Akhdar, Faisal, Giza, FAISAL</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1484,37 +1480,41 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/675289</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/673329</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>El Eslamboly Co. For Air Condition, Cooling &amp; Import</t>
+          <t>El Fath For Paints</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0235688202</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
+          <t>01156551455</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>01156551455</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>71 El Ekhwa Tower, El Mahatta St., Floor 1, Giza, Giza, GIZA</t>
+          <t>9 Refaah St., Mansheyet El Bakry, Heliopolis, Cairo, HELIOPOLIS</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>مواد البناء والمقاولات</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>☎ هاتف فقط</t>
+          <t>📱 واتساب فقط</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1524,36 +1524,36 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/351285</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/556559</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>El Esnawy For Computer Supplies</t>
+          <t>Abdel Wahab For Building Materials</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>01013660278</t>
+          <t>01006567538</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>01013660278</t>
+          <t>01006567538</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>7 Madraset El Motafaweqin St., Ain shams, Cairo, AIN SHAMS</t>
+          <t>26 Abnaa Sohag St., Imbaba, Giza, IMBABA</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>مواد البناء والمقاولات</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1568,41 +1568,37 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/622831</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/580008</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Zeyad Silver</t>
+          <t>MB Group For Cooling Towers</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>01015909052</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>01015909052</t>
-        </is>
-      </c>
+          <t>0226237471</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Mahaleya 6, , 1st District, Obour city, Kaliobeya, OBOUR CITY</t>
+          <t>84 Joseph Tito St., Highkestep, Cairo, HIGHKESTEP</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>التكييف والتبريد</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>📱 واتساب فقط</t>
+          <t>☎ هاتف فقط</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1612,33 +1608,41 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/525984</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/375122</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Brickzey</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
+          <t>Trweeg</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>01200100522</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>01200100522</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Customer Service, El Sheikh Zayed, 6th of october, Giza, 6th OF OCTOBER</t>
+          <t>6 Dory Abaza St.El Zohour District, El zagazig, El sharkeya, EL ZAGAZIG</t>
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>العقارات والمقاولات</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>📱 واتساب فقط</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1648,36 +1652,36 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/589092</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/631436</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Betna</t>
+          <t>El Alameya For Sanitary Ware</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>01287412222</t>
+          <t>01006463407</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>01287412222</t>
+          <t>01006463407</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Misr Ismaileya Desert Rd., Golf City, Obour city, Kaliobeya, OBOUR CITY</t>
+          <t>50 Petrol St., Ezbet El Hafir, El khosous, Kaliobeya, EL KHOSOUS</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1692,30 +1696,30 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/505820</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/500815</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Babay</t>
+          <t>Khaled El Fayoumi For Foods</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>01271872131</t>
+          <t>01110121540</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>01271872131</t>
+          <t>01110121540</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>50 Ahmed Zaky St., Hadayek El Maadi, Maadi, Cairo, MAADI</t>
+          <t>., 6th District, 6th of october, Giza, 6th OF OCTOBER</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1736,36 +1740,36 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/334829</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/437230</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Clinic Labs</t>
+          <t>Dr. Abdel Nasser Awad Center</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>01096598537</t>
+          <t>01111017450</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>01096598537</t>
+          <t>01111017450</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>El Madina El Monawara St., El Fardous, 6th of october, Giza, 6th OF OCTOBER</t>
+          <t>Km 21 Sq., Agami, Alexandria, AGAMI</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>المعدات الطبية والصيدلانية</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1780,41 +1784,37 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/611816</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/487818</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Fresco Restaurant &amp; Cafe</t>
+          <t>El Roumany Laundry</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>01032703370</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>01032703370</t>
-        </is>
-      </c>
+          <t>0224300059</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2 Palestine St., El Maadi Complex, New Maadi, Maadi, Cairo, MAADI</t>
+          <t>22 Meniet El Serg St., Shoubra, Cairo, SHOUBRA</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>الأغذية والمشروبات</t>
+          <t>أدوات النظافة</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>📱 واتساب فقط</t>
+          <t>☎ هاتف فقط</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1824,30 +1824,30 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/635133</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/467242</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Bait El Monsef Restaurant</t>
+          <t>SE Data For Computer Maintenance</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>01156451400</t>
+          <t>01227051766</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>01156451400</t>
+          <t>01227051766</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>., 7th District, 6th of october, Giza, 6th OF OCTOBER</t>
+          <t>, Central Spine, 6th of october, Giza, 6th OF OCTOBER</t>
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
@@ -1868,37 +1868,33 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/446146</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/487044</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Tabalina Cafe &amp; Restaurant</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>0233375988</t>
-        </is>
-      </c>
+          <t>Dr. Hazem Mahmoud</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>16 Abdel Aziz Selim St.  Off El Thawra St., Mohandeseen, Giza, MOHANDESEEN</t>
+          <t>Aly Mobarak St.  Intersection Of El Nady St., Tanta, El gharbeya, TANTA</t>
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>الأغذية والمشروبات</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>☎ هاتف فقط</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -1908,36 +1904,36 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/585069</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/592074</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Abraj City For Real Estate Marketing</t>
+          <t>El Farouq</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>01030969643</t>
+          <t>01066216340</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>01030969643</t>
+          <t>01066216340</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>, El Yasmeen 7, Villa 2, 5th Compound, New cairo, Cairo, NEW CAIRO</t>
+          <t>34 Mostafa Kamel St., Hadayek El Maadi, Maadi, Cairo, MAADI</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1952,37 +1948,41 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/696727</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/417231</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Tono For Clothes</t>
+          <t>Abdel Fatah For Advertising</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0237614616</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
+          <t>01004734121</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>01004734121</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>42 Abdel Moneim Riad St., Off El Batal Ahmed Abdel Aziz St., Mohandeseen, Giza, MOHANDESEEN</t>
+          <t>8 Abdel Rahman Amin St., Off Ibrahim Abdel Razeq St., Ain shams el sharkeya, Cairo, AIN SHAMS EL SHARKEYA</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>النسيج والملابس</t>
+          <t>الطباعة والنشر والإعلان</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>☎ هاتف فقط</t>
+          <t>📱 واتساب فقط</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -1992,36 +1992,36 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/590467</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/652127</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Sara Clean</t>
+          <t>Express Security Systems</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>01008277809</t>
+          <t>01002213386</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>01008277809</t>
+          <t>01002213386</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Mansour El Sanadily St., Faisal, Giza, FAISAL</t>
+          <t>, El Ordoneya, 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>أدوات النظافة</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2036,36 +2036,36 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/417755</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/693390</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Designo Furniture</t>
+          <t>Hebeish Medical</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>01116840670</t>
+          <t>01280383699</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>01116840670</t>
+          <t>01280383699</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>12 Taha Hussein St.  El Moalemeen Division, Hadayek helwan, Cairo, HADAYEK HELWAN</t>
+          <t>10 El Naggar St., El sayeda zeinab, Cairo, EL SAYEDA ZEINAB</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>المعدات الطبية والصيدلانية</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2080,36 +2080,36 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/597155</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/704958</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>el Tahawy For Medical Supplies</t>
+          <t>Sun Center Cleaning</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>01016155000</t>
+          <t>01142751314</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>01016155000</t>
+          <t>01142751314</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>11 el sheikh aly youssef st., Mounira, Cairo, MOUNIRA</t>
+          <t>4 Rd. 104, Maadi, Cairo, MAADI</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>المعدات الطبية والصيدلانية</t>
+          <t>أدوات النظافة</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2124,37 +2124,41 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/621918</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/505699</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Attaby Lab</t>
+          <t>Cottonil</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0228516480</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr"/>
+          <t>01150535500</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>01150535500</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>14 Amin Yousry St.  Off El Kanisa El Faransawy St., Ezbet el nakhl, Cairo, EZBET EL NAKHL</t>
+          <t>2 Mohamed Abdullah St., Shoubra el khaymah, Kaliobeya, SHOUBRA EL KHAYMAH</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>المعدات الطبية والصيدلانية</t>
+          <t>النسيج والملابس</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>☎ هاتف فقط</t>
+          <t>📱 واتساب فقط</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2164,37 +2168,41 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/527152</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/413462</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Aga Comprehensive Clinic</t>
+          <t>Faisal For Clothes</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0504458848</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
+          <t>01282684757</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>01282684757</t>
+        </is>
+      </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>El Baylouk District, Aga, El dakahleya, AGA</t>
+          <t>4 El Sayeda Aaesha St., Tukh, Kaliobeya, TUKH</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>تكنولوجيا المعلومات (IT)</t>
+          <t>النسيج والملابس</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>☎ هاتف فقط</t>
+          <t>📱 واتساب فقط</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2204,36 +2212,36 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/363770</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/515729</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Me For Clothes</t>
+          <t>Ashram Chemicals - Dr. Soheb Basam Al Ashram</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>01007309007</t>
+          <t>01000007187</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>01007309007</t>
+          <t>01000007187</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1 Petroleum Bldgs., Ahmed Orabi St., Mohandeseen, Giza, MOHANDESEEN</t>
+          <t>3rd Industrial Zone B3, 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>النسيج والملابس</t>
+          <t>مواد البناء والمقاولات</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2248,41 +2256,37 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/463890</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/592016</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Technical Workshop For Cars Maintenance</t>
+          <t>El Shefaa Specialized Clinics</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>01220296176</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>01220296176</t>
-        </is>
-      </c>
+          <t>0227774287</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1 Ouda Rady St., El marg, Cairo, EL MARG</t>
+          <t>30 Abdel Hamid Othman St., Ain shams, Cairo, AIN SHAMS</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>السيارات وقطع الغيار</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>📱 واتساب فقط</t>
+          <t>☎ هاتف فقط</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2292,36 +2296,36 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/561948</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/325434</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Dakar</t>
+          <t>Bazin Furniture</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>01148580098</t>
+          <t>01005277458</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>01148580098</t>
+          <t>01005277458</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>30 Borhan St., Intersection Of Haidar St., Helwan, Cairo, HELWAN</t>
+          <t>5 Asaad Gomaa St., Damietta, Damietta, DAMIETTA</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>النسيج والملابس</t>
+          <t>الأثاث المكتبي</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2336,26 +2340,30 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/384288</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/505983</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>El Masreya For Computer</t>
+          <t>El Rawda Air Condition</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>0224983875</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr"/>
+          <t>01002061996</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>01002061996</t>
+        </is>
+      </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>70 Ain Shams St., Ain shams el sharkeya, Cairo, AIN SHAMS EL SHARKEYA</t>
+          <t>., 6th of october, Giza, 6th OF OCTOBER</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -2366,7 +2374,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>☎ هاتف فقط</t>
+          <t>📱 واتساب فقط</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2376,36 +2384,36 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/661421</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/436827</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Dice Underwear</t>
+          <t>Online For Computer</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>01212095539</t>
+          <t>01027962524</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>01212095539</t>
+          <t>01027962524</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1 Kaabish St., Intersection Of Arbaeen St., El Tawabeq, Faisal, Giza, FAISAL</t>
+          <t>49 Noubar St., Bab el louk, Cairo, BAB EL LOUK</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>النسيج والملابس</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2420,41 +2428,37 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/397953</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/618619</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Abdel Halim For Cars Plumping</t>
+          <t>Kimo Sat</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>01002071698</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>01002071698</t>
-        </is>
-      </c>
+          <t>0464901736</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>49 Amin El Gendy  St., Zahraa Ain Shams, Ain shams, Cairo, AIN SHAMS</t>
+          <t>Km 7, , Bldg. 41, Matrouh alex. desert rd., North coast, MATROUH ALEX. DESERT RD.</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>السيارات وقطع الغيار</t>
+          <t>تكنولوجيا المعلومات (IT)</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>📱 واتساب فقط</t>
+          <t>☎ هاتف فقط</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2464,41 +2468,33 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/661121</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/583233</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Raya7 Balak</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>01157845959</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>01157845959</t>
-        </is>
-      </c>
+          <t>Carrefour Market</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>28 El Falaky St., Downtown, Cairo, DOWNTOWN</t>
+          <t>34 El Mostashfa St., Shoubra, Cairo, SHOUBRA</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>معدات المطابخ الكبيرة الفندقية وقطع غيارها</t>
+          <t>الأغذية والمشروبات</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>📱 واتساب فقط</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2508,36 +2504,36 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/675297</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/703046</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Khater Sons Furniture</t>
+          <t>El Ayouty Dairy</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>01201376127</t>
+          <t>01224902009</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>01201376127</t>
+          <t>01224902009</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>7 Ard El Maared St., Tanan Village, Qalyub, Kaliobeya, QALYUB</t>
+          <t>21 Salah El Din St., Bab El Haras, Damietta, Damietta, DAMIETTA</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>الأثاث المكتبي</t>
+          <t>الأغذية والمشروبات</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2552,51 +2548,2179 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/519476</t>
+          <t>https://www.yellowpages.com.eg/en/profile/x/503499</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Aqua Roza For Water Treatment</t>
+          <t>Benaya &amp; Aman</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>01201362417</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>01201362417</t>
-        </is>
-      </c>
+          <t>0889182297</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>8 Bekhit Hawary St., Shoubra, Cairo, SHOUBRA</t>
+          <t>El Wataneya Towers El Gomhoreya St., Assyout, Assyout, Assyout</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
+          <t>مواد البناء والمقاولات</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>☎ هاتف فقط</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/671449</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Patio Office Furniture</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>01008944703</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>01008944703</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>3 Aly El Gendy St., Off Ahmed Fakhry St., Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/680766</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Dixon's Restaurant</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>01020819513</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>01020819513</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>51 Kafr Abdou St., Roushdy, Alexandria, ROUSHDY</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>الأغذية والمشروبات</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/469897</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>El Floka Seafood</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>01113776007</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>01113776007</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Km 33, Cairo Suez Desert Rd., Madinty, Cairo, Madinty</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>الأغذية والمشروبات</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/572605</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>El Amana For Electrical Appliances Maintenance</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>01221846155</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>01221846155</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>6 El Madina El Monawara St., Warraq El Arab, El warak, Giza, EL WARAK</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/595219</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Horse White Coffee Shop</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>01124433491</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>01124433491</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>42 Sherif Pasha St., Helwan, Cairo, HELWAN</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/643164</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Sun Switch</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>01211118771</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>01211118771</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>19 Demascus St., Mohandeseen, Giza, MOHANDESEEN</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/490029</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Souk El Asr For Women Clothes</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>01018804401</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>01018804401</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>45 Port Said St., El shohadaa, El monofeya, El Shohadaa</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>النسيج والملابس</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/547708</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>El Shagra El Tayba Charitable</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>01006070136</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>01006070136</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Abou Bakr El Seddik St., El Ordoneya, 10th of ramadan, El sharkeya, 10th OF RAMADAN</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/619627</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Alaa For Food</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>0222500871</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>5 West El Balad St., Ain shams el gharbeya, Cairo, AIN SHAMS EL GHARBEYA</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>الأغذية والمشروبات</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>☎ هاتف فقط</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/535165</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>N N For Sanitary Ware</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>01004623293</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>01004623293</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>13 El Madina El Monawara St., Saft El Laban, Boulak el dakrour, Giza, BOULAK EL DAKROUR</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/575868</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Water Engineering For Pumps Assembly</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>01122414848</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>01122414848</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Plot 61, 1st Industrial Zone, Sadat city, El monofeya, SADAT City</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
           <t>معالجة المياه والصرف الصحي</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>📱 واتساب فقط</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>YellowPages</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>https://www.yellowpages.com.eg/en/profile/x/669541</t>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/684746</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Mabaret Al Asafra Laboratories</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>El Horreya Rd., Sporting, Alexandria, SPORTING</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>المعدات الطبية والصيدلانية</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/713424</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Mohamed El Omda For Electrical Appliances</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>01110449995</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>01110449995</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>33 Teraet El Sawahel St., Geziret Mohamed Village, El warak, Giza, EL WARAK</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/600033</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Sun City Tours</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>01024488418</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>01024488418</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>12 302 st., Semouha, Alexandria, SEMOUHA</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/622024</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Joint Clinic - Dr. Ibrahim Gado For Orthopedic &amp; Joints</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>01111191169</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>01111191169</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>305 Shoubra St., Floor 2, Shoubra, Cairo, SHOUBRA</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/605583</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Ashraf Abou Ahmed For Electrical Supplies</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>01100628380</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>01100628380</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>7 Hussein Gad El Rab St., El Gezirah, Dar el salam, Cairo, DAR EL SALAM</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/499011</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Koky For Kids Wear</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>01016145855</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>01016145855</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>29 Hasab Allah El Kafrawy St., 2nd District Center, New damietta, Damietta, NEW DAMIETTA</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>النسيج والملابس</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/528929</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>El Anwar For Electrical Appliances</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>01152669455</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>01152669455</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>1 Ard El Sherif St., El Awqaf Bldg., Abdin, Cairo, ABDIN</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/648924</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>El Marwa Workshop For Blacksmithing</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>01112093239</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>01112093239</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>68 Kamal Hegab St., Mansheyet El Sad El Aaly, Gesr el suez, Cairo, GESR EL SUEZ</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/453553</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Silver Town</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>01222428671</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>01222428671</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Ring Rd., New cairo, Cairo, NEW CAIRO</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/708170</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Legend For Print</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>01003260885</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>01003260885</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>3 Sekket El Saraiga St., El kalag, Kaliobeya, EL KALAG</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>الطباعة والنشر والإعلان</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/515016</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Aqua Treat</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>01110055628</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>01110055628</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>11 Aly Shalaby St., Farid Semeika St., Hegaz Square, Heliopolis, Cairo, HELIOPOLIS</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>معالجة المياه والصرف الصحي</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/621375</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>5 Roosters Fried Chicken</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>41 Abdel Hamid Badawy St., Off Soteir St., Azarita, Alexandria, AZARITA</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>الأغذية والمشروبات</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/663311</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Fathalla Market</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Km 56, Alex. matrouh desert rd., North coast, ALEX. MATROUH DESERT RD.</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>الأغذية والمشروبات</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/689343</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>El Raya For Real Estate Development</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>01112220716</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>01112220716</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>27 el tayaran st., Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>العقارات والمقاولات</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/313943</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>El Hamd For Steel And Cement Trade</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>01289280051</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>01289280051</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>, 5th Zone, Sadat city, El monofeya, SADAT City</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>مواد البناء والمقاولات</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/709462</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Classy Furniture</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>01224106249</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>01224106249</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>40 Abdel Razeq Gawhar St., Ard el lewaa, Giza, Ard El Lewaa</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>الأثاث المكتبي</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/551563</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>El Omda For Metalworks</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>01155564777</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>01155564777</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>70 Aly Salama St., El Manawat, Giza, Giza, GIZA</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>الميكانيكا</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/616911</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Sharkasia Restaurant</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>0224736797</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>8 Africa St., Extension Of Mostafa El Nahhas St., Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>الأغذية والمشروبات</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>☎ هاتف فقط</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/469656</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Fathet Khair For Vegetables &amp; Fruits</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>01030196463</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>01030196463</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>26 Sayed Saleh St., Faisal, Giza, FAISAL</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/685143</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>McDonald's</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Plot 67/68, 1st District Services Zone, 5th Compound, New cairo, Cairo, NEW CAIRO</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>الأغذية والمشروبات</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/449324</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Nour El Hoda For Electrical Tools</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>01282705530</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>01282705530</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>2 Said Aly St., Ain shams el gharbeya, Cairo, AIN SHAMS EL GHARBEYA</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/657986</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Panorama Electric For Engineering Industries</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>0238890095</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Plot 102,   Extension Of 6th Zone, Industrial Zone, 6th of october, Giza, 6th OF OCTOBER</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>الكهرباء والكابلات والأسلاك</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>☎ هاتف فقط</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/512804</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Afaaq</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>0227543111</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>11 W/5 Menshawy St.  Off El Nasr St., New Maadi, Maadi, Cairo, MAADI</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>الميكانيكا</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>☎ هاتف فقط</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/457883</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>United Establishment For General Supplies</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>01061486898</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>01061486898</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>17 Bostan El Dekka St., Off Emad El Din St., Downtown, Cairo, DOWNTOWN</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/691314</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Panee Take Away</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>01091885269</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>01091885269</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>11 A Arab Organization For Industrialization Bldgs.,, Nasr city, Cairo, NASR CITY</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>الأغذية والمشروبات</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/457630</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Serget Nada</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>01271770662</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>01271770662</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>20 Masged El Shahed St., Kerdasa, Giza, Kerdasa</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>الأغذية والمشروبات</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/557956</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Rewaa For Import &amp; Export</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>0222661410</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Square 1258Z, Bldg. 1S,   Extension Of Abdel Hamid Badawy St., Sheraton Bldgs., Heliopolis, Cairo, HELIOPOLIS</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>النسيج والملابس</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>☎ هاتف فقط</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/553194</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Amer Real Estate Marketing</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>01020307434</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>01020307434</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>105 B Gehaz El Madina St., 4th District, 5th Compound, New cairo, Cairo, NEW CAIRO</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>الطباعة والنشر والإعلان</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/614886</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Yehia For Clothes</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>01011608787</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>01011608787</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>2 El Nozha St., Hadayek El Maadi, Maadi, Cairo, MAADI</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>النسيج والملابس</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/675807</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Seboua</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>0572320069</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>35 El Noqrashy St., Damietta, Damietta, DAMIETTA</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>الأغذية والمشروبات</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>☎ هاتف فقط</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/505515</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Trust Smart Systems</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>035855160</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>360 El Guish Rd., Glim, Alexandria, GLIM</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>☎ هاتف فقط</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/450223</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Ziko Play Station</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>01150276082</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>01150276082</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>29 Ahmed Badawy St., Kafr El Shorafa, El marg, Cairo, EL MARG</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/565193</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Al Fagr For Engineering Works</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>01122243330</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>01122243330</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>18 K, Hadayek El Ahram, El haram, Giza, EL HARAM</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>مواد البناء والمقاولات</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/630352</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Danash Bakery</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>01152992568</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>01152992568</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>El Mostashfa El Markazy St., El khanka, Kaliobeya, EL KHANKA</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>الأغذية والمشروبات</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/415467</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Mohamed Tolba For Clothes Supplies</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>01114054130</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>01114054130</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>7 Abnaa Sohag St., Saft El Laban, Boulak el dakrour, Giza, BOULAK EL DAKROUR</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>النسيج والملابس</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/576169</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>ESLA</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>01270705044</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>01270705044</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>, Phase 3, Al rehab city, Cairo, AL REHAB CITY</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>النسيج والملابس</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/527090</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Mas Relocation &amp; Real Estate</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>0223583863</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>61 El Canal St., Maadi, Cairo, MAADI</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>العقارات والمقاولات</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>☎ هاتف فقط</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/420847</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Rotary</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>01026164648</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>01026164648</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Momtaz Ghoraba St.  Intersection Of Hassan Ibn Thabet St., Tanta, El gharbeya, TANTA</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>الأغذية والمشروبات</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>📱 واتساب فقط</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/582425</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Nour Sat For Dish</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>0228456088</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>264 El Nasr Bldgs.,, Mokattam, Cairo, MOKATTAM</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>تكنولوجيا المعلومات (IT)</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>☎ هاتف فقط</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>YellowPages</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>https://www.yellowpages.com.eg/en/profile/x/441262</t>
         </is>
       </c>
     </row>

</xml_diff>